<commit_message>
update draft & ref
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pva/work/github.com/doclang-project/doclang-standard/spec_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pva/work/github.com/doclang-project/doclang-standard/reference/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20275C91-6688-6C40-BD6C-9C8359044E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28754C19-F5E3-8E4B-9A4E-13888C8D69FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1600" yWindow="500" windowWidth="33300" windowHeight="28300" activeTab="1" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
+    <workbookView xWindow="-34560" yWindow="7220" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="4" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">attributes!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">elements!$A$1:$H$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">elements!$A$1:$H$76</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="182">
   <si>
     <t>{"read_only", "fillable"}</t>
   </si>
@@ -83,9 +83,6 @@
     <t>[01b] semantic (inner)</t>
   </si>
   <si>
-    <t>[02] grouping</t>
-  </si>
-  <si>
     <t>[05] formatting</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
     <t>Is attribute required</t>
   </si>
   <si>
-    <t>Scoping of a field key (optional) &amp; any corresponding values.</t>
-  </si>
-  <si>
     <t>The key of a field (may correspond to  0-N field values).</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
     <t>`&lt;field_region&gt;`</t>
   </si>
   <si>
-    <t>`&lt;otsl&gt;`</t>
-  </si>
-  <si>
     <t>`&lt;list&gt;`</t>
   </si>
   <si>
@@ -170,9 +161,6 @@
     <t>`&lt;marker&gt;`</t>
   </si>
   <si>
-    <t>`&lt;list_text&gt;`</t>
-  </si>
-  <si>
     <t>`&lt;field_heading&gt;`</t>
   </si>
   <si>
@@ -368,9 +356,6 @@
     <t>Contains a `&lt;uri&gt;` and then optionally raw or formatted text data.</t>
   </si>
   <si>
-    <t>Can only be child of `&lt;otsl&gt;`.</t>
-  </si>
-  <si>
     <t>`value`</t>
   </si>
   <si>
@@ -393,10 +378,6 @@
   </si>
   <si>
     <t>`h_thread_id`</t>
-  </si>
-  <si>
-    <t>needed?
-Yes, if the individual hour/minute/etc are not all required (else cannot unambiguously interpret `&lt;hour&gt;0&lt;/hour&gt;&lt;minute&gt;2&lt;/minute&gt;&lt;second&gt;3&lt;/second&gt;`)</t>
   </si>
   <si>
     <t>Allowed attribute values</t>
@@ -515,9 +496,6 @@
     <t>Any context that allows semantic elements.</t>
   </si>
   <si>
-    <t>Any context that allows grouping elements.</t>
-  </si>
-  <si>
     <t>Payload elements are low-level elements that help define the effective content of another element.</t>
   </si>
   <si>
@@ -542,9 +520,6 @@
     <t>[Content] Raw text</t>
   </si>
   <si>
-    <t>Can only be child of a semantic or a grouping element (or of `&lt;otsl&gt;` in the context of "implicit `&lt;text&gt;`s").</t>
-  </si>
-  <si>
     <t>Grouping elements enable the encapsulation of semantic elements or other grouping elements. Any grouping element may optionally begin with a [component head](#component-head-elements).</t>
   </si>
   <si>
@@ -552,9 +527,6 @@
   </si>
   <si>
     <t>Element Description</t>
-  </si>
-  <si>
-    <t>Captures a table using OTSL format. A table cell, as delimited  by the respective structural elements, can be defined either by normal semantic / grouping elements or by an optional component head followed by raw or formatted text, which is to be interpreted as an "implicit `&lt;text&gt;`" (i.e. without the wrapping tags).</t>
   </si>
   <si>
     <t>The component head is a sequence comprising the following elements in this order, whereby all elements are optional:&lt;br /&gt;&lt;ul&gt;&lt;li&gt;`&lt;thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;h_thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;meta&gt;`&lt;/li&gt;&lt;li&gt;sequence of 2*N `&lt;location&gt;`s (N&gt;1)&lt;/li&gt;&lt;li&gt;sequence of `&lt;timestamp&gt;`s&lt;/li&gt;&lt;li&gt;`&lt;layer&gt;`&lt;/li&gt;&lt;/ul&gt;
@@ -562,15 +534,6 @@
 The various component head elements are further specified in the following subsections.</t>
   </si>
   <si>
-    <t>[TODO: revise] Container that groups a floating component with its caption, footnotes etc.</t>
-  </si>
-  <si>
-    <t>[Content] Semantic / grouping elements</t>
-  </si>
-  <si>
-    <t>[TODO: revise] Generic container to be used for grouping mixed-type components.</t>
-  </si>
-  <si>
     <t>Any context that allows raw text content.</t>
   </si>
   <si>
@@ -591,6 +554,45 @@
   </si>
   <si>
     <t>The document root element. Starts with an optional `&lt;head&gt;` followed by a sequence of applicable elements.</t>
+  </si>
+  <si>
+    <t>TBD. Needed, if the individual hour/minute/etc are not all required (else cannot unambiguously interpret `&lt;hour&gt;0&lt;/hour&gt;&lt;minute&gt;2&lt;/minute&gt;&lt;second&gt;3&lt;/second&gt;`)</t>
+  </si>
+  <si>
+    <t>`&lt;table&gt;`</t>
+  </si>
+  <si>
+    <t>Can only be child of `&lt;table&gt;`.</t>
+  </si>
+  <si>
+    <t>Delimiter defining the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
+  </si>
+  <si>
+    <t>`&lt;ld&gt;`</t>
+  </si>
+  <si>
+    <t>Captures a list. List items are delimited by the respective structural elements.</t>
+  </si>
+  <si>
+    <t>[01] semantic (top)</t>
+  </si>
+  <si>
+    <t>Container for encapsulating multiple semantic elements.</t>
+  </si>
+  <si>
+    <t>[Content] Semantic elements</t>
+  </si>
+  <si>
+    <t>Can only be child of a semantic element.</t>
+  </si>
+  <si>
+    <t>Only `&lt;marker&gt;`</t>
+  </si>
+  <si>
+    <t>Captures a table based on the OTSL format. Table cells are delimited by the respective structural elements.</t>
+  </si>
+  <si>
+    <t>Scoping of a field key (optional) and any corresponding values.</t>
   </si>
 </sst>
 </file>
@@ -1007,74 +1009,74 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B4" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B7" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B9" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1084,7 +1086,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986C0F9C-DD53-344B-9F2F-F3D5821A4A0E}">
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.1640625" style="2" bestFit="1" customWidth="1"/>
@@ -1104,22 +1106,22 @@
         <v>7</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1127,10 +1129,10 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>9</v>
@@ -1153,13 +1155,13 @@
         <v>10</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E3" s="6" t="b">
         <v>1</v>
@@ -1179,13 +1181,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E4" s="6" t="b">
         <v>0</v>
@@ -1205,13 +1207,13 @@
         <v>11</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E5" s="6" t="b">
         <v>1</v>
@@ -1231,11 +1233,11 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E6" s="6" t="b">
         <v>1</v>
@@ -1259,7 +1261,7 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E7" s="6" t="b">
         <v>1</v>
@@ -1279,11 +1281,11 @@
         <v>11</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E8" s="6" t="b">
         <v>1</v>
@@ -1303,11 +1305,11 @@
         <v>11</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E9" s="6" t="b">
         <v>1</v>
@@ -1327,11 +1329,11 @@
         <v>11</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E10" s="6" t="b">
         <v>1</v>
@@ -1351,11 +1353,13 @@
         <v>11</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="D11" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E11" s="6" t="b">
         <v>1</v>
@@ -1364,24 +1368,24 @@
         <v>1</v>
       </c>
       <c r="G11" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>35</v>
+        <v>170</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>17</v>
+        <v>180</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E12" s="6" t="b">
         <v>1</v>
@@ -1396,18 +1400,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E13" s="6" t="b">
         <v>1</v>
@@ -1415,8 +1419,8 @@
       <c r="F13" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="G13" s="6" t="b">
-        <v>1</v>
+      <c r="G13" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H13" s="1" t="b">
         <v>1</v>
@@ -1427,11 +1431,11 @@
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E14" s="6" t="b">
         <v>1</v>
@@ -1440,10 +1444,10 @@
         <v>1</v>
       </c>
       <c r="G14" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1451,11 +1455,11 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E15" s="6" t="b">
         <v>1</v>
@@ -1475,11 +1479,11 @@
         <v>11</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E16" s="6" t="b">
         <v>1</v>
@@ -1488,10 +1492,10 @@
         <v>1</v>
       </c>
       <c r="G16" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1499,11 +1503,11 @@
         <v>11</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E17" s="6" t="b">
         <v>1</v>
@@ -1512,7 +1516,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="1" t="b">
         <v>1</v>
@@ -1520,14 +1524,16 @@
     </row>
     <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>11</v>
+        <v>175</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="5"/>
+        <v>44</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>176</v>
+      </c>
       <c r="D18" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E18" s="6" t="b">
         <v>1</v>
@@ -1536,22 +1542,22 @@
         <v>1</v>
       </c>
       <c r="G18" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E19" s="6" t="b">
         <v>1</v>
@@ -1571,11 +1577,13 @@
         <v>12</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>181</v>
+      </c>
       <c r="D20" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E20" s="6" t="b">
         <v>1</v>
@@ -1584,7 +1592,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="1" t="b">
         <v>1</v>
@@ -1595,13 +1603,13 @@
         <v>12</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E21" s="6" t="b">
         <v>1</v>
@@ -1610,7 +1618,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" s="1" t="b">
         <v>1</v>
@@ -1621,13 +1629,13 @@
         <v>12</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E22" s="6" t="b">
         <v>1</v>
@@ -1647,271 +1655,265 @@
         <v>12</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E23" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+      <c r="A24" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E23" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F23" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G23" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E24" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A25" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E24" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G24" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H24" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>48</v>
-      </c>
       <c r="C25" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>156</v>
+        <v>119</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>178</v>
       </c>
       <c r="E25" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" s="1" t="b">
         <v>0</v>
       </c>
       <c r="H25" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E26" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E26" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G26" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H26" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="153" x14ac:dyDescent="0.2">
-      <c r="A27" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E27" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G27" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E27" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F27" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G27" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H27" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A28" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E28" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H28" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E28" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F28" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G28" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A29" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E29" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F29" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H29" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E29" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F29" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G29" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H29" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A30" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5"/>
+      <c r="D30" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E30" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F30" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E30" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F30" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G30" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H30" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A31" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="5"/>
+      <c r="D31" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E31" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F31" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G31" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H31" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E31" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F31" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G31" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H31" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A32" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5"/>
+      <c r="D32" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H32" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E32" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H32" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A33" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>56</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="6" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="E33" s="6" t="b">
         <v>0</v>
@@ -1926,16 +1928,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="E34" s="6" t="b">
         <v>0</v>
@@ -1950,73 +1952,75 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E35" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G35" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H35" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A36" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E35" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F35" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G35" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H35" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A36" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="5"/>
+      <c r="D36" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E36" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F36" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H36" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A37" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="5"/>
-      <c r="D36" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E36" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F36" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G36" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H36" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A37" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="6" t="s">
-        <v>165</v>
+      <c r="C37" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="E37" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G37" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H37" s="1" t="b">
         <v>0</v>
@@ -2024,23 +2028,23 @@
     </row>
     <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>105</v>
+        <v>162</v>
       </c>
       <c r="E38" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G38" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" s="1" t="b">
         <v>0</v>
@@ -2048,14 +2052,14 @@
     </row>
     <row r="39" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>105</v>
+        <v>162</v>
       </c>
       <c r="E39" s="6" t="b">
         <v>1</v>
@@ -2070,18 +2074,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>120</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="E40" s="6" t="b">
         <v>1</v>
@@ -2089,7 +2091,7 @@
       <c r="F40" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G40" s="1" t="b">
+      <c r="G40" s="6" t="b">
         <v>1</v>
       </c>
       <c r="H40" s="1" t="b">
@@ -2098,23 +2100,23 @@
     </row>
     <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E41" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G41" s="1" t="b">
-        <v>0</v>
+      <c r="G41" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H41" s="1" t="b">
         <v>0</v>
@@ -2122,14 +2124,14 @@
     </row>
     <row r="42" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E42" s="6" t="b">
         <v>1</v>
@@ -2137,7 +2139,7 @@
       <c r="F42" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G42" s="1" t="b">
+      <c r="G42" s="6" t="b">
         <v>1</v>
       </c>
       <c r="H42" s="1" t="b">
@@ -2146,14 +2148,14 @@
     </row>
     <row r="43" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E43" s="6" t="b">
         <v>1</v>
@@ -2165,19 +2167,19 @@
         <v>1</v>
       </c>
       <c r="H43" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E44" s="6" t="b">
         <v>1</v>
@@ -2189,19 +2191,19 @@
         <v>1</v>
       </c>
       <c r="H44" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E45" s="6" t="b">
         <v>1</v>
@@ -2213,19 +2215,19 @@
         <v>1</v>
       </c>
       <c r="H45" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E46" s="6" t="b">
         <v>1</v>
@@ -2237,43 +2239,47 @@
         <v>1</v>
       </c>
       <c r="H46" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E47" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G47" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H47" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A48" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E47" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F47" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G47" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H47" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A48" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C48" s="5"/>
+      <c r="C48" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="D48" s="5" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E48" s="6" t="b">
         <v>1</v>
@@ -2285,7 +2291,7 @@
         <v>1</v>
       </c>
       <c r="H48" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -2293,23 +2299,23 @@
         <v>14</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E49" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F49" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G49" s="6" t="b">
-        <v>1</v>
+      <c r="G49" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H49" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -2317,63 +2323,59 @@
         <v>14</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>121</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E50" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F50" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G50" s="6" t="b">
-        <v>1</v>
+      <c r="G50" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H50" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>107</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E51" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F51" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G51" s="6" t="b">
-        <v>1</v>
+      <c r="G51" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H51" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E52" s="6" t="b">
         <v>0</v>
@@ -2390,14 +2392,14 @@
     </row>
     <row r="53" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E53" s="6" t="b">
         <v>0</v>
@@ -2414,14 +2416,14 @@
     </row>
     <row r="54" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E54" s="6" t="b">
         <v>0</v>
@@ -2438,14 +2440,14 @@
     </row>
     <row r="55" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E55" s="6" t="b">
         <v>0</v>
@@ -2462,14 +2464,14 @@
     </row>
     <row r="56" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E56" s="6" t="b">
         <v>0</v>
@@ -2486,14 +2488,14 @@
     </row>
     <row r="57" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E57" s="6" t="b">
         <v>0</v>
@@ -2510,14 +2512,14 @@
     </row>
     <row r="58" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="E58" s="6" t="b">
         <v>0</v>
@@ -2532,19 +2534,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C59" s="5"/>
+        <v>173</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>172</v>
+      </c>
       <c r="D59" s="5" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E59" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F59" s="6" t="b">
         <v>0</v>
@@ -2552,64 +2556,68 @@
       <c r="G59" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H59" s="1" t="b">
-        <v>0</v>
+      <c r="H59" s="1" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>15</v>
+        <v>144</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E60" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F60" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G60" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H60" s="1" t="b">
-        <v>0</v>
+        <v>26</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>15</v>
+        <v>144</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H61" s="1" t="b">
-        <v>0</v>
+        <v>81</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>5</v>
@@ -2632,10 +2640,10 @@
     </row>
     <row r="63" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>5</v>
@@ -2658,10 +2666,10 @@
     </row>
     <row r="64" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>5</v>
@@ -2684,10 +2692,10 @@
     </row>
     <row r="65" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>5</v>
@@ -2710,10 +2718,10 @@
     </row>
     <row r="66" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>5</v>
@@ -2736,10 +2744,10 @@
     </row>
     <row r="67" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>5</v>
@@ -2762,10 +2770,10 @@
     </row>
     <row r="68" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>5</v>
@@ -2788,10 +2796,10 @@
     </row>
     <row r="69" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>5</v>
@@ -2814,10 +2822,10 @@
     </row>
     <row r="70" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>5</v>
@@ -2840,10 +2848,10 @@
     </row>
     <row r="71" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>5</v>
@@ -2866,10 +2874,10 @@
     </row>
     <row r="72" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>5</v>
@@ -2892,10 +2900,10 @@
     </row>
     <row r="73" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>5</v>
@@ -2918,10 +2926,10 @@
     </row>
     <row r="74" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>5</v>
@@ -2944,10 +2952,10 @@
     </row>
     <row r="75" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>5</v>
@@ -2970,10 +2978,10 @@
     </row>
     <row r="76" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>5</v>
@@ -2994,70 +3002,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A77" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="B77" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D77" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E77" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F77" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G77" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H77" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A78" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="B78" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D78" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F78" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G78" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A79" s="1"/>
-      <c r="B79" s="1"/>
-      <c r="C79" s="1"/>
-      <c r="D79" s="1"/>
-      <c r="F79" s="1"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A80" s="4"/>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A77" s="1"/>
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="F77" s="1"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A78" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H78" xr:uid="{986C0F9C-DD53-344B-9F2F-F3D5821A4A0E}"/>
+  <autoFilter ref="A1:H76" xr:uid="{986C0F9C-DD53-344B-9F2F-F3D5821A4A0E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3080,145 +3036,145 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
       <c r="D1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="E2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" t="s">
         <v>139</v>
-      </c>
-      <c r="D4" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="D5" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D6" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D7" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D8" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D9" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -3226,13 +3182,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C11" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D11" t="s">
         <v>0</v>
@@ -3240,13 +3196,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B12" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D12" t="s">
         <v>3</v>
@@ -3254,13 +3210,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
@@ -3268,27 +3224,27 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
@@ -3296,33 +3252,33 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D16" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E16" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D17" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
document versioning management, switch to v0
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pva/work/github.com/doclang-project/doclang-standard/reference/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B9AADE-4221-DA43-891F-CF491583F188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A814EF-C50D-004B-948D-8458FD1A3094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="4" r:id="rId1"/>
@@ -439,12 +439,6 @@
     <t>structural</t>
   </si>
   <si>
-    <t xml:space="preserve">The DocLang specification version the document was produced against. </t>
-  </si>
-  <si>
-    <t>Optional; default: "1.0.0"</t>
-  </si>
-  <si>
     <t>Required</t>
   </si>
   <si>
@@ -466,9 +460,6 @@
     <t>Integer within [0, resolution)</t>
   </si>
   <si>
-    <t>In format "x.y.z" as per Semantic Versioning</t>
-  </si>
-  <si>
     <t>Postive integer</t>
   </si>
   <si>
@@ -479,12 +470,6 @@
   </si>
   <si>
     <t>[07] document head</t>
-  </si>
-  <si>
-    <t>Optional; default: "https://www.doclang.ai/ns/v1"</t>
-  </si>
-  <si>
-    <t>{"https://www.doclang.ai/ns/v1"}</t>
   </si>
   <si>
     <t xml:space="preserve">The DocLang specification version namespace. </t>
@@ -593,6 +578,21 @@
   </si>
   <si>
     <t>`&lt;ldiv&gt;`</t>
+  </si>
+  <si>
+    <t>Optional; default: "0.1"</t>
+  </si>
+  <si>
+    <t>Optional; default: "https://www.doclang.ai/ns/v0"</t>
+  </si>
+  <si>
+    <t>{"https://www.doclang.ai/ns/v0"}</t>
+  </si>
+  <si>
+    <t>{"0.1"}</t>
+  </si>
+  <si>
+    <t>The DocLang specification version the document is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Verisoning.</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1020,7 @@
         <v>125</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="85" x14ac:dyDescent="0.2">
@@ -1036,7 +1036,7 @@
         <v>126</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="102" x14ac:dyDescent="0.2">
@@ -1044,7 +1044,7 @@
         <v>127</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -1052,7 +1052,7 @@
         <v>128</v>
       </c>
       <c r="B6" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -1060,7 +1060,7 @@
         <v>129</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -1068,15 +1068,15 @@
         <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B9" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1106,22 +1106,22 @@
         <v>7</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1132,7 +1132,7 @@
         <v>23</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>9</v>
@@ -1184,7 +1184,7 @@
         <v>24</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>96</v>
@@ -1210,10 +1210,10 @@
         <v>28</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E5" s="6" t="b">
         <v>1</v>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E6" s="6" t="b">
         <v>1</v>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E7" s="6" t="b">
         <v>1</v>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E8" s="6" t="b">
         <v>1</v>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E9" s="6" t="b">
         <v>1</v>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E10" s="6" t="b">
         <v>1</v>
@@ -1359,7 +1359,7 @@
         <v>16</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E11" s="6" t="b">
         <v>1</v>
@@ -1379,13 +1379,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E12" s="6" t="b">
         <v>1</v>
@@ -1408,10 +1408,10 @@
         <v>34</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E13" s="6" t="b">
         <v>1</v>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E14" s="6" t="b">
         <v>1</v>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E15" s="6" t="b">
         <v>1</v>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E16" s="6" t="b">
         <v>1</v>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E17" s="6" t="b">
         <v>1</v>
@@ -1524,16 +1524,16 @@
     </row>
     <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E18" s="6" t="b">
         <v>1</v>
@@ -1580,7 +1580,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>99</v>
@@ -1684,10 +1684,10 @@
         <v>46</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E24" s="6" t="b">
         <v>0</v>
@@ -1713,7 +1713,7 @@
         <v>119</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E25" s="6" t="b">
         <v>0</v>
@@ -1736,10 +1736,10 @@
         <v>48</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E26" s="6" t="b">
         <v>1</v>
@@ -1765,7 +1765,7 @@
         <v>22</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E27" s="6" t="b">
         <v>1</v>
@@ -1791,7 +1791,7 @@
         <v>120</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E28" s="6" t="b">
         <v>0</v>
@@ -1814,10 +1814,10 @@
         <v>51</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E29" s="6" t="b">
         <v>1</v>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E30" s="6" t="b">
         <v>0</v>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E31" s="6" t="b">
         <v>0</v>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E32" s="6" t="b">
         <v>0</v>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E33" s="6" t="b">
         <v>0</v>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E34" s="6" t="b">
         <v>0</v>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E38" s="6" t="b">
         <v>0</v>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E39" s="6" t="b">
         <v>1</v>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E40" s="6" t="b">
         <v>1</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E41" s="6" t="b">
         <v>1</v>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E42" s="6" t="b">
         <v>1</v>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E43" s="6" t="b">
         <v>1</v>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E44" s="6" t="b">
         <v>1</v>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E45" s="6" t="b">
         <v>1</v>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E46" s="6" t="b">
         <v>1</v>
@@ -2253,7 +2253,7 @@
         <v>115</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E47" s="6" t="b">
         <v>1</v>
@@ -2279,7 +2279,7 @@
         <v>103</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E48" s="6" t="b">
         <v>1</v>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E49" s="6" t="b">
         <v>0</v>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E50" s="6" t="b">
         <v>0</v>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E51" s="6" t="b">
         <v>0</v>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E52" s="6" t="b">
         <v>0</v>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E53" s="6" t="b">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E54" s="6" t="b">
         <v>0</v>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E55" s="6" t="b">
         <v>0</v>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E56" s="6" t="b">
         <v>0</v>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E57" s="6" t="b">
         <v>0</v>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E58" s="6" t="b">
         <v>0</v>
@@ -2539,10 +2539,10 @@
         <v>14</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>98</v>
@@ -2557,12 +2557,12 @@
         <v>0</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>26</v>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="61" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>81</v>
@@ -2614,7 +2614,7 @@
     </row>
     <row r="62" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>82</v>
@@ -2640,7 +2640,7 @@
     </row>
     <row r="63" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>83</v>
@@ -2666,7 +2666,7 @@
     </row>
     <row r="64" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>84</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="65" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>85</v>
@@ -2718,7 +2718,7 @@
     </row>
     <row r="66" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>86</v>
@@ -2744,7 +2744,7 @@
     </row>
     <row r="67" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>87</v>
@@ -2770,7 +2770,7 @@
     </row>
     <row r="68" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>57</v>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="69" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>88</v>
@@ -2822,7 +2822,7 @@
     </row>
     <row r="70" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>89</v>
@@ -2848,7 +2848,7 @@
     </row>
     <row r="71" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>90</v>
@@ -2874,7 +2874,7 @@
     </row>
     <row r="72" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>91</v>
@@ -2900,7 +2900,7 @@
     </row>
     <row r="73" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>92</v>
@@ -2926,7 +2926,7 @@
     </row>
     <row r="74" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>93</v>
@@ -2952,7 +2952,7 @@
     </row>
     <row r="75" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>94</v>
@@ -2978,7 +2978,7 @@
     </row>
     <row r="76" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>95</v>
@@ -3053,16 +3053,16 @@
         <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>145</v>
+        <v>178</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
+        <v>179</v>
       </c>
       <c r="E2" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -3073,13 +3073,13 @@
         <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>132</v>
+        <v>177</v>
       </c>
       <c r="D3" t="s">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="E3" t="s">
-        <v>131</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -3090,10 +3090,10 @@
         <v>104</v>
       </c>
       <c r="C4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -3104,10 +3104,10 @@
         <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -3118,10 +3118,10 @@
         <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -3132,10 +3132,10 @@
         <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -3146,10 +3146,10 @@
         <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D8" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -3160,10 +3160,10 @@
         <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -3174,7 +3174,7 @@
         <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -3188,7 +3188,7 @@
         <v>108</v>
       </c>
       <c r="C11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D11" t="s">
         <v>0</v>
@@ -3202,7 +3202,7 @@
         <v>108</v>
       </c>
       <c r="C12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D12" t="s">
         <v>3</v>
@@ -3216,7 +3216,7 @@
         <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
@@ -3230,7 +3230,7 @@
         <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D14" t="s">
         <v>15</v>
@@ -3244,7 +3244,7 @@
         <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
@@ -3258,13 +3258,13 @@
         <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D16" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E16" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -3275,10 +3275,10 @@
         <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D17" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: align lists, tables, groups, headings
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pva/work/github.com/doclang-project/doclang-standard/reference/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E5F33BA-4BB4-1B4A-9E0B-B0223A046B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2844DA7-CF56-C642-9073-E85B6EB95CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="179">
   <si>
     <t>{"read_only", "fillable"}</t>
   </si>
@@ -50,9 +50,6 @@
     <t>{"unordered", "ordered"}</t>
   </si>
   <si>
-    <t>{"false", "true"}</t>
-  </si>
-  <si>
     <t>{"code", "formula", "picture"}</t>
   </si>
   <si>
@@ -366,9 +363,6 @@
   </si>
   <si>
     <t>`class`</t>
-  </si>
-  <si>
-    <t>`selected`</t>
   </si>
   <si>
     <t>`thread_id`</t>
@@ -439,9 +433,6 @@
     <t>Optional; defaults to head metadata `&lt;default_resolution&gt;`, otherwise "512"</t>
   </si>
   <si>
-    <t>Optional;default: "false"</t>
-  </si>
-  <si>
     <t>Optional; default: "unordered"</t>
   </si>
   <si>
@@ -587,6 +578,12 @@
   </si>
   <si>
     <t>Includes doc-level metadata. Also discussed in Appendix B.</t>
+  </si>
+  <si>
+    <t>{"unselected", "selected"}</t>
+  </si>
+  <si>
+    <t>Optional; default: "unselected"</t>
   </si>
 </sst>
 </file>
@@ -1003,66 +1000,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="85" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1086,42 +1083,42 @@
   <sheetData>
     <row r="1" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>7</v>
-      </c>
       <c r="C1" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2" s="6" t="b">
         <v>1</v>
@@ -1138,16 +1135,16 @@
     </row>
     <row r="3" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E3" s="6" t="b">
         <v>1</v>
@@ -1164,16 +1161,16 @@
     </row>
     <row r="4" spans="1:8" ht="136" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E4" s="6" t="b">
         <v>0</v>
@@ -1190,16 +1187,16 @@
     </row>
     <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E5" s="6" t="b">
         <v>1</v>
@@ -1216,14 +1213,14 @@
     </row>
     <row r="6" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E6" s="6" t="b">
         <v>1</v>
@@ -1240,14 +1237,14 @@
     </row>
     <row r="7" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E7" s="6" t="b">
         <v>1</v>
@@ -1264,14 +1261,14 @@
     </row>
     <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E8" s="6" t="b">
         <v>1</v>
@@ -1288,14 +1285,14 @@
     </row>
     <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E9" s="6" t="b">
         <v>1</v>
@@ -1312,14 +1309,14 @@
     </row>
     <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E10" s="6" t="b">
         <v>1</v>
@@ -1336,16 +1333,16 @@
     </row>
     <row r="11" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E11" s="6" t="b">
         <v>1</v>
@@ -1362,16 +1359,16 @@
     </row>
     <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E12" s="6" t="b">
         <v>1</v>
@@ -1388,16 +1385,16 @@
     </row>
     <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E13" s="6" t="b">
         <v>1</v>
@@ -1414,14 +1411,14 @@
     </row>
     <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E14" s="6" t="b">
         <v>1</v>
@@ -1438,14 +1435,14 @@
     </row>
     <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E15" s="6" t="b">
         <v>1</v>
@@ -1462,14 +1459,14 @@
     </row>
     <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E16" s="6" t="b">
         <v>1</v>
@@ -1486,14 +1483,14 @@
     </row>
     <row r="17" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E17" s="6" t="b">
         <v>1</v>
@@ -1510,16 +1507,16 @@
     </row>
     <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E18" s="6" t="b">
         <v>1</v>
@@ -1536,14 +1533,14 @@
     </row>
     <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E19" s="6" t="b">
         <v>1</v>
@@ -1560,16 +1557,16 @@
     </row>
     <row r="20" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E20" s="6" t="b">
         <v>1</v>
@@ -1586,16 +1583,16 @@
     </row>
     <row r="21" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E21" s="6" t="b">
         <v>1</v>
@@ -1612,16 +1609,16 @@
     </row>
     <row r="22" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E22" s="6" t="b">
         <v>1</v>
@@ -1638,16 +1635,16 @@
     </row>
     <row r="23" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E23" s="6" t="b">
         <v>1</v>
@@ -1664,16 +1661,16 @@
     </row>
     <row r="24" spans="1:8" ht="153" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E24" s="6" t="b">
         <v>0</v>
@@ -1690,16 +1687,16 @@
     </row>
     <row r="25" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E25" s="6" t="b">
         <v>0</v>
@@ -1716,16 +1713,16 @@
     </row>
     <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E26" s="6" t="b">
         <v>1</v>
@@ -1742,16 +1739,16 @@
     </row>
     <row r="27" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E27" s="6" t="b">
         <v>1</v>
@@ -1768,16 +1765,16 @@
     </row>
     <row r="28" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E28" s="6" t="b">
         <v>0</v>
@@ -1794,16 +1791,16 @@
     </row>
     <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E29" s="6" t="b">
         <v>1</v>
@@ -1820,14 +1817,14 @@
     </row>
     <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E30" s="6" t="b">
         <v>0</v>
@@ -1844,14 +1841,14 @@
     </row>
     <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E31" s="6" t="b">
         <v>0</v>
@@ -1868,14 +1865,14 @@
     </row>
     <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E32" s="6" t="b">
         <v>0</v>
@@ -1892,14 +1889,14 @@
     </row>
     <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E33" s="6" t="b">
         <v>0</v>
@@ -1916,14 +1913,14 @@
     </row>
     <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E34" s="6" t="b">
         <v>0</v>
@@ -1940,14 +1937,14 @@
     </row>
     <row r="35" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E35" s="6" t="b">
         <v>1</v>
@@ -1964,14 +1961,14 @@
     </row>
     <row r="36" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E36" s="6" t="b">
         <v>1</v>
@@ -1988,16 +1985,16 @@
     </row>
     <row r="37" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E37" s="6" t="b">
         <v>1</v>
@@ -2014,14 +2011,14 @@
     </row>
     <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E38" s="6" t="b">
         <v>0</v>
@@ -2038,14 +2035,14 @@
     </row>
     <row r="39" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E39" s="6" t="b">
         <v>1</v>
@@ -2062,14 +2059,14 @@
     </row>
     <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E40" s="6" t="b">
         <v>1</v>
@@ -2086,14 +2083,14 @@
     </row>
     <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E41" s="6" t="b">
         <v>1</v>
@@ -2110,14 +2107,14 @@
     </row>
     <row r="42" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E42" s="6" t="b">
         <v>1</v>
@@ -2134,14 +2131,14 @@
     </row>
     <row r="43" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E43" s="6" t="b">
         <v>1</v>
@@ -2158,14 +2155,14 @@
     </row>
     <row r="44" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E44" s="6" t="b">
         <v>1</v>
@@ -2182,14 +2179,14 @@
     </row>
     <row r="45" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E45" s="6" t="b">
         <v>1</v>
@@ -2206,14 +2203,14 @@
     </row>
     <row r="46" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E46" s="6" t="b">
         <v>1</v>
@@ -2230,16 +2227,16 @@
     </row>
     <row r="47" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E47" s="6" t="b">
         <v>1</v>
@@ -2256,16 +2253,16 @@
     </row>
     <row r="48" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E48" s="6" t="b">
         <v>1</v>
@@ -2282,14 +2279,14 @@
     </row>
     <row r="49" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E49" s="6" t="b">
         <v>0</v>
@@ -2306,14 +2303,14 @@
     </row>
     <row r="50" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E50" s="6" t="b">
         <v>0</v>
@@ -2330,14 +2327,14 @@
     </row>
     <row r="51" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E51" s="6" t="b">
         <v>0</v>
@@ -2354,14 +2351,14 @@
     </row>
     <row r="52" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E52" s="6" t="b">
         <v>0</v>
@@ -2378,14 +2375,14 @@
     </row>
     <row r="53" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E53" s="6" t="b">
         <v>0</v>
@@ -2402,14 +2399,14 @@
     </row>
     <row r="54" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E54" s="6" t="b">
         <v>0</v>
@@ -2426,14 +2423,14 @@
     </row>
     <row r="55" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E55" s="6" t="b">
         <v>0</v>
@@ -2450,14 +2447,14 @@
     </row>
     <row r="56" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E56" s="6" t="b">
         <v>0</v>
@@ -2474,14 +2471,14 @@
     </row>
     <row r="57" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E57" s="6" t="b">
         <v>0</v>
@@ -2498,14 +2495,14 @@
     </row>
     <row r="58" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E58" s="6" t="b">
         <v>0</v>
@@ -2522,16 +2519,16 @@
     </row>
     <row r="59" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E59" s="6" t="b">
         <v>1</v>
@@ -2543,449 +2540,449 @@
         <v>0</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
@@ -3019,162 +3016,162 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
       <c r="D1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D3" t="s">
         <v>172</v>
       </c>
-      <c r="D3" t="s">
-        <v>175</v>
-      </c>
       <c r="E3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D11" t="s">
         <v>0</v>
@@ -3182,27 +3179,27 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
@@ -3210,61 +3207,61 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>131</v>
+        <v>178</v>
       </c>
       <c r="D15" t="s">
-        <v>2</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D16" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E16" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D17" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add virtual text support to lists and tables, incl. validation
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pva/work/github.com/doclang-project/doclang-standard/reference/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2844DA7-CF56-C642-9073-E85B6EB95CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C3EA8C-E00B-5142-B418-E517FB1E412A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
+    <workbookView xWindow="25280" yWindow="3480" windowWidth="34560" windowHeight="21580" activeTab="2" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="193">
   <si>
     <t>{"read_only", "fillable"}</t>
   </si>
@@ -496,9 +496,6 @@
     <t>Any context that allows raw text content.</t>
   </si>
   <si>
-    <t>Represents a piece of cohesive text as that would appear in a paragraph.</t>
-  </si>
-  <si>
     <t>Indicates a page break. A paginated document may be divided into pages using the `&lt;page_break/&gt;` empty element. Any page content, as split by `&lt;page_break/&gt;`, forms a valid DocLang [document body](#head-and-body-areas), i.e. would be a valid DocLang document if wrapped in a `doclang` root element.</t>
   </si>
   <si>
@@ -524,12 +521,6 @@
     <t>Can only be child of `&lt;table&gt;`.</t>
   </si>
   <si>
-    <t>Delimiter defining the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
-  </si>
-  <si>
-    <t>Captures a list. List items are delimited by the respective structural elements.</t>
-  </si>
-  <si>
     <t>[01] semantic (top)</t>
   </si>
   <si>
@@ -545,25 +536,16 @@
     <t>Only `&lt;marker&gt;`</t>
   </si>
   <si>
-    <t>Captures a table based on the OTSL format. Table cells are delimited by the respective structural elements.</t>
-  </si>
-  <si>
     <t>Scoping of a field key (optional) and any corresponding values.</t>
   </si>
   <si>
     <t>`&lt;ldiv&gt;`</t>
   </si>
   <si>
-    <t>Optional; default: "0.1"</t>
-  </si>
-  <si>
     <t>Optional; default: "https://www.doclang.ai/ns/v0"</t>
   </si>
   <si>
     <t>{"https://www.doclang.ai/ns/v0"}</t>
-  </si>
-  <si>
-    <t>{"0.1"}</t>
   </si>
   <si>
     <t>The DocLang specification version the document is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Verisoning.</t>
@@ -584,6 +566,66 @@
   </si>
   <si>
     <t>Optional; default: "unselected"</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of an empty cell.</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of a column header cell.</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of a row header cell.</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of a section row header.</t>
+  </si>
+  <si>
+    <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+  </si>
+  <si>
+    <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+  </si>
+  <si>
+    <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
+  </si>
+  <si>
+    <t>New line / new table row</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of a full / regular cell.</t>
+  </si>
+  <si>
+    <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
+  </si>
+  <si>
+    <t>`level`</t>
+  </si>
+  <si>
+    <t>Optional; default "1"</t>
+  </si>
+  <si>
+    <t>{"0.2"}</t>
+  </si>
+  <si>
+    <t>Optional; default: "0.2"</t>
+  </si>
+  <si>
+    <t>Represents a piece of cohesive text as that would appear in a paragraph. Note: a special construct related to this element is the so-called "virtual `&lt;text&gt;`", which can occur only as a list item or a table cell — see `&lt;list&gt;` and `&lt;table&gt;` below for details.</t>
+  </si>
+  <si>
+    <t>Captures a list. List items are delimited by the respective structural elements. A list item can be defined without a wrapping tag, i.e. as pure (optional) component head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRUE, also on cell level in case of virtual `&lt;text&gt;` </t>
+  </si>
+  <si>
+    <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+  </si>
+  <si>
+    <t>Captures a table, in a format inspired by OTSL. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) component head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1069,7 @@
         <v>123</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1051,7 +1093,7 @@
         <v>126</v>
       </c>
       <c r="B7" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -1104,7 +1146,7 @@
         <v>146</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1115,7 +1157,7 @@
         <v>21</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1141,7 +1183,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>95</v>
@@ -1167,7 +1209,7 @@
         <v>22</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>94</v>
@@ -1185,7 +1227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
@@ -1193,7 +1235,7 @@
         <v>26</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>139</v>
@@ -1357,15 +1399,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>157</v>
+        <v>32</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>139</v>
@@ -1373,25 +1415,25 @@
       <c r="E12" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="F12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" s="1" t="b">
-        <v>0</v>
+      <c r="F12" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="H12" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>160</v>
+        <v>192</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>139</v>
@@ -1399,11 +1441,11 @@
       <c r="E13" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="F13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="1" t="b">
-        <v>0</v>
+      <c r="F13" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="H13" s="1" t="b">
         <v>1</v>
@@ -1507,13 +1549,13 @@
     </row>
     <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>42</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>139</v>
@@ -1563,7 +1605,7 @@
         <v>38</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>97</v>
@@ -1667,10 +1709,10 @@
         <v>44</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E24" s="6" t="b">
         <v>0</v>
@@ -1696,7 +1738,7 @@
         <v>116</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E25" s="6" t="b">
         <v>0</v>
@@ -1719,10 +1761,10 @@
         <v>46</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E26" s="6" t="b">
         <v>1</v>
@@ -1748,7 +1790,7 @@
         <v>20</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E27" s="6" t="b">
         <v>1</v>
@@ -1774,7 +1816,7 @@
         <v>117</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E28" s="6" t="b">
         <v>0</v>
@@ -1797,10 +1839,10 @@
         <v>49</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E29" s="6" t="b">
         <v>1</v>
@@ -1824,7 +1866,7 @@
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E30" s="6" t="b">
         <v>0</v>
@@ -1848,7 +1890,7 @@
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E31" s="6" t="b">
         <v>0</v>
@@ -1872,7 +1914,7 @@
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E32" s="6" t="b">
         <v>0</v>
@@ -1896,7 +1938,7 @@
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E33" s="6" t="b">
         <v>0</v>
@@ -1920,7 +1962,7 @@
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E34" s="6" t="b">
         <v>0</v>
@@ -2284,9 +2326,11 @@
       <c r="B49" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C49" s="5"/>
+      <c r="C49" s="5" t="s">
+        <v>182</v>
+      </c>
       <c r="D49" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E49" s="6" t="b">
         <v>0</v>
@@ -2308,9 +2352,11 @@
       <c r="B50" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C50" s="5"/>
+      <c r="C50" s="5" t="s">
+        <v>173</v>
+      </c>
       <c r="D50" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E50" s="6" t="b">
         <v>0</v>
@@ -2332,9 +2378,11 @@
       <c r="B51" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C51" s="5"/>
+      <c r="C51" s="5" t="s">
+        <v>174</v>
+      </c>
       <c r="D51" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E51" s="6" t="b">
         <v>0</v>
@@ -2356,9 +2404,11 @@
       <c r="B52" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C52" s="5"/>
+      <c r="C52" s="5" t="s">
+        <v>175</v>
+      </c>
       <c r="D52" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E52" s="6" t="b">
         <v>0</v>
@@ -2373,16 +2423,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C53" s="5"/>
+      <c r="C53" s="5" t="s">
+        <v>176</v>
+      </c>
       <c r="D53" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E53" s="6" t="b">
         <v>0</v>
@@ -2404,9 +2456,11 @@
       <c r="B54" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C54" s="5"/>
+      <c r="C54" s="5" t="s">
+        <v>177</v>
+      </c>
       <c r="D54" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E54" s="6" t="b">
         <v>0</v>
@@ -2421,16 +2475,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C55" s="5"/>
+      <c r="C55" s="5" t="s">
+        <v>178</v>
+      </c>
       <c r="D55" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E55" s="6" t="b">
         <v>0</v>
@@ -2445,16 +2501,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C56" s="5"/>
+      <c r="C56" s="5" t="s">
+        <v>179</v>
+      </c>
       <c r="D56" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E56" s="6" t="b">
         <v>0</v>
@@ -2469,16 +2527,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C57" s="5"/>
+      <c r="C57" s="5" t="s">
+        <v>180</v>
+      </c>
       <c r="D57" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E57" s="6" t="b">
         <v>0</v>
@@ -2500,9 +2560,11 @@
       <c r="B58" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C58" s="5"/>
+      <c r="C58" s="5" t="s">
+        <v>181</v>
+      </c>
       <c r="D58" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E58" s="6" t="b">
         <v>0</v>
@@ -2522,10 +2584,10 @@
         <v>12</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>159</v>
+        <v>183</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>96</v>
@@ -2540,7 +2602,7 @@
         <v>0</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -3004,7 +3066,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD42BB9-A54F-044A-A968-54A6AE9BC2F8}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
@@ -3039,10 +3101,10 @@
         <v>138</v>
       </c>
       <c r="C2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D2" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E2" t="s">
         <v>137</v>
@@ -3056,13 +3118,13 @@
         <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="D3" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="E3" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -3165,102 +3227,116 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>184</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>185</v>
       </c>
       <c r="D11" t="s">
-        <v>0</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
         <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D12" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>103</v>
       </c>
       <c r="B13" t="s">
         <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D13" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B14" t="s">
         <v>106</v>
       </c>
       <c r="C14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s">
         <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>178</v>
+        <v>127</v>
       </c>
       <c r="D15" t="s">
-        <v>177</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" t="s">
+        <v>172</v>
+      </c>
+      <c r="D16" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>44</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>107</v>
-      </c>
-      <c r="C16" t="s">
-        <v>127</v>
-      </c>
-      <c r="D16" t="s">
-        <v>133</v>
-      </c>
-      <c r="E16" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" t="s">
-        <v>108</v>
       </c>
       <c r="C17" t="s">
         <v>127</v>
       </c>
       <c r="D17" t="s">
+        <v>133</v>
+      </c>
+      <c r="E17" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" t="s">
+        <v>127</v>
+      </c>
+      <c r="D18" t="s">
         <v>133</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add cross-reference support, refactor hyperlink support
- Replace `<uri>` with `<src>` in `<picture>` elements across the documentation.
- Introduce `<xref>` and `<href>` elements in the component head, enforcing mutual exclusivity.
- Update validation rules to ensure proper placement of `<xref>` and `<href>`.
- Remove deprecated `<hyperlink>` element and related test cases.
- Add new test cases for validating `<href>` and `<xref>` usage.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -11,10 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$10</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -538,7 +538,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>The component head is a sequence comprising the following elements in this order, whereby all elements are optional:&lt;br /&gt;&lt;ul&gt;&lt;li&gt;`&lt;thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;h_thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;meta&gt;`&lt;/li&gt;&lt;li&gt;sequence of 2*N `&lt;location&gt;`s (N&gt;1)&lt;/li&gt;&lt;li&gt;sequence of `&lt;timestamp&gt;`s&lt;/li&gt;&lt;li&gt;`&lt;layer&gt;`&lt;/li&gt;&lt;/ul&gt;
+          <t>The component head is a sequence comprising the following elements in this order, whereby all elements are optional:&lt;br /&gt;&lt;ul&gt;&lt;li&gt;`&lt;thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;h_thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;xref&gt;` or `&lt;href&gt;` (mutually exclusive)&lt;/li&gt;&lt;li&gt;`&lt;meta&gt;`&lt;/li&gt;&lt;li&gt;sequence of 2*N `&lt;location&gt;`s (N&gt;1)&lt;/li&gt;&lt;li&gt;sequence of `&lt;timestamp&gt;`s&lt;/li&gt;&lt;li&gt;`&lt;layer&gt;`&lt;/li&gt;&lt;/ul&gt;
 A component head can only appear as the leading content of a semantic element.
 The various component head elements are further specified in the following subsections.</t>
         </is>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -612,7 +612,8 @@
     <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="10"/>
+    <col width="20" customWidth="1" style="1" min="11" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1442,7 +1443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="34" customHeight="1">
+    <row r="26" ht="68" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>[03a] component head (outer)</t>
@@ -1450,21 +1451,21 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>`&lt;meta&gt;`</t>
+          <t>`&lt;xref&gt;`</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Used to store additional or derived information regarding the respective component.</t>
+          <t>Optional part of the component head; serves for capturing an outgoing cross-reference from this component.</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;href&gt;`.</t>
         </is>
       </c>
       <c r="E26" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="6" t="b">
         <v>0</v>
@@ -1484,17 +1485,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>`&lt;custom_meta&gt;`</t>
+          <t>`&lt;href&gt;`</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Custom metadata, e.g. for application-specific purposes.</t>
+          <t>Optional part of the component head; serves for capturing a URI referenced by this component.</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;xref&gt;`.</t>
         </is>
       </c>
       <c r="E27" s="6" t="b">
@@ -1504,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" s="1" t="b">
         <v>0</v>
@@ -1516,117 +1517,125 @@
           <t>[03a] component head (outer)</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;meta&gt;`</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Used to store additional or derived information regarding the respective component.</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H28" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>[03a] component head (outer)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;custom_meta&gt;`</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Custom metadata, e.g. for application-specific purposes.</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F29" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H29" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>[03a] component head (outer)</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>`&lt;location&gt;`</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Coordinate system is the bottom-left corner of the page.</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
         </is>
       </c>
-      <c r="E28" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F28" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G28" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" ht="85" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="E30" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F30" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" ht="85" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>[03a] component head (outer)</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>`&lt;timestamp&gt;`</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>TBD. Needed, if the individual hour/minute/etc are not all required (else cannot unambiguously interpret `&lt;hour&gt;0&lt;/hour&gt;&lt;minute&gt;2&lt;/minute&gt;&lt;second&gt;3&lt;/second&gt;`)</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F29" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G29" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H29" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>[03a] component head (outer)</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;hour&gt;`</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F30" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G30" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H30" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" ht="17" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>[03a] component head (outer)</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;minute&gt;`</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
       <c r="E31" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" s="6" t="b">
         <v>0</v>
@@ -1646,7 +1655,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>`&lt;second&gt;`</t>
+          <t>`&lt;hour&gt;`</t>
         </is>
       </c>
       <c r="C32" s="5" t="n"/>
@@ -1676,7 +1685,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>`&lt;centisecond&gt;`</t>
+          <t>`&lt;minute&gt;`</t>
         </is>
       </c>
       <c r="C33" s="5" t="n"/>
@@ -1706,7 +1715,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>`&lt;layer&gt;`</t>
+          <t>`&lt;second&gt;`</t>
         </is>
       </c>
       <c r="C34" s="5" t="n"/>
@@ -1731,28 +1740,28 @@
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>[03b] component head (inner)</t>
+          <t>[03a] component head (outer)</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;centisecond&gt;`</t>
         </is>
       </c>
       <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;meta&gt;`.</t>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
         </is>
       </c>
       <c r="E35" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G35" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" s="1" t="b">
         <v>0</v>
@@ -1761,52 +1770,48 @@
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
+          <t>[03a] component head (outer)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;layer&gt;`</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H36" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
           <t>[03b] component head (inner)</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;classification&gt;`</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;summary&gt;`</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;meta&gt;`.</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F36" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G36" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H36" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>[04] payload</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;uri&gt;`</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Textual content must be a URI.</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;picture&gt;` or first child of `&lt;hyperlink&gt;`.</t>
         </is>
       </c>
       <c r="E37" s="6" t="b">
@@ -1825,34 +1830,34 @@
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>[04] payload</t>
+          <t>[03b] component head (inner)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
+          <t>`&lt;classification&gt;`</t>
         </is>
       </c>
       <c r="C38" s="5" t="n"/>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be child of `&lt;meta&gt;`.</t>
         </is>
       </c>
       <c r="E38" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G38" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="17" customHeight="1">
+    <row r="39" ht="34" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
@@ -1860,23 +1865,27 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>`&lt;content&gt;`</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="n"/>
+          <t>`&lt;src&gt;`</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>The image's source.</t>
+        </is>
+      </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be child of `&lt;picture&gt;`.</t>
         </is>
       </c>
       <c r="E39" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G39" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" s="1" t="b">
         <v>0</v>
@@ -1885,12 +1894,12 @@
     <row r="40" ht="17" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="C40" s="5" t="n"/>
@@ -1900,13 +1909,13 @@
         </is>
       </c>
       <c r="E40" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G40" s="6" t="b">
-        <v>1</v>
+      <c r="G40" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H40" s="1" t="b">
         <v>0</v>
@@ -1915,12 +1924,12 @@
     <row r="41" ht="17" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
+          <t>`&lt;content&gt;`</t>
         </is>
       </c>
       <c r="C41" s="5" t="n"/>
@@ -1935,7 +1944,7 @@
       <c r="F41" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G41" s="6" t="b">
+      <c r="G41" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H41" s="1" t="b">
@@ -1950,7 +1959,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
+          <t>`&lt;bold&gt;`</t>
         </is>
       </c>
       <c r="C42" s="5" t="n"/>
@@ -1980,7 +1989,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
+          <t>`&lt;italic&gt;`</t>
         </is>
       </c>
       <c r="C43" s="5" t="n"/>
@@ -2010,7 +2019,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
+          <t>`&lt;underline&gt;`</t>
         </is>
       </c>
       <c r="C44" s="5" t="n"/>
@@ -2040,7 +2049,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
+          <t>`&lt;strikethrough&gt;`</t>
         </is>
       </c>
       <c r="C45" s="5" t="n"/>
@@ -2070,7 +2079,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
+          <t>`&lt;superscript&gt;`</t>
         </is>
       </c>
       <c r="C46" s="5" t="n"/>
@@ -2100,14 +2109,10 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Indicates right-to-left direction.</t>
-        </is>
-      </c>
+          <t>`&lt;subscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="n"/>
       <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2126,7 +2131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" ht="34" customHeight="1">
+    <row r="48" ht="17" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
           <t>[05] formatting</t>
@@ -2134,14 +2139,10 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;hyperlink&gt;`</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Contains a `&lt;uri&gt;` and then optionally raw or formatted text data.</t>
-        </is>
-      </c>
+          <t>`&lt;handwriting&gt;`</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="n"/>
       <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2163,32 +2164,32 @@
     <row r="49" ht="17" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;rtl&gt;`</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates right-to-left direction.</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E49" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G49" s="1" t="b">
-        <v>0</v>
+      <c r="G49" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H49" s="1" t="b">
         <v>0</v>
@@ -2202,12 +2203,12 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -2236,12 +2237,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2270,311 +2271,303 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
+          <t>`&lt;ched&gt;`</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a column header cell.</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`.</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F52" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G52" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H52" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="17" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
           <t>`&lt;rhed&gt;`</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a row header cell.</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E52" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F52" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G52" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H52" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" ht="34" customHeight="1">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="E53" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F53" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G53" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H53" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" ht="34" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>`&lt;corn&gt;`</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E53" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F53" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G53" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H53" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" ht="17" customHeight="1">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="E54" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F54" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G54" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H54" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" ht="17" customHeight="1">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>`&lt;srow&gt;`</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a section row header.</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E54" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F54" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G54" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H54" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" ht="51" customHeight="1">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="E55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H55" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" ht="51" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>`&lt;lcel&gt;`</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E55" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F55" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G55" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H55" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" ht="34" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="E56" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H56" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" ht="34" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>`&lt;ucel&gt;`</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E56" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F56" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G56" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H56" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" ht="51" customHeight="1">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="E57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G57" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H57" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" ht="51" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E57" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F57" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G57" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H57" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" ht="17" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="E58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="17" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>`&lt;nl&gt;`</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>New line / new table row</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`.</t>
         </is>
       </c>
-      <c r="E58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G58" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H58" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="34" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="E59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" ht="34" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>`&lt;ldiv&gt;`</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;list&gt;`.</t>
         </is>
       </c>
-      <c r="E59" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="inlineStr">
+      <c r="E60" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H60" s="1" t="inlineStr">
         <is>
           <t>Only `&lt;marker&gt;`</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="17" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>[07] document head</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;title&gt;`</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2579,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
+          <t>`&lt;title&gt;`</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2628,7 +2621,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -2670,7 +2663,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -2712,7 +2705,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2754,7 +2747,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2796,7 +2789,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -2838,7 +2831,7 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -2880,7 +2873,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -2922,7 +2915,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -2964,7 +2957,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3006,7 +2999,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3048,7 +3041,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3090,7 +3083,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3132,7 +3125,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3174,7 +3167,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;access_policy&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3216,52 +3209,94 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
+          <t>`&lt;retention_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="17" customHeight="1">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
           <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
-      <c r="C76" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="1" t="n"/>
-      <c r="B77" s="1" t="n"/>
-      <c r="C77" s="1" t="n"/>
-      <c r="D77" s="1" t="n"/>
-      <c r="F77" s="1" t="n"/>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="n"/>
+      <c r="A78" s="1" t="n"/>
+      <c r="B78" s="1" t="n"/>
+      <c r="C78" s="1" t="n"/>
+      <c r="D78" s="1" t="n"/>
+      <c r="F78" s="1" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H76"/>
+  <autoFilter ref="A1:H77"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3273,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3404,7 +3439,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Postive integer</t>
+          <t>Positive integer</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3730,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Postive integer</t>
+          <t>Positive integer</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3722,7 +3757,88 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Postive integer</t>
+          <t>Positive integer</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>`&lt;xref&gt;`</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>`thread_id`</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>The ID of the referenced thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>`&lt;href&gt;`</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>`uri`</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>The URI of the referenced resource.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>`&lt;src&gt;`</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>`uri`</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>The source URI.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor terminology, move `<caption>` to element head
- Update documentation to replace references from "component head" to "element head" throughout the schema and related files.
- Clarify the structure of semantic elements, emphasizing the separation of properties and content.
- Introduce new validation rules and examples to ensure proper placement of properties like `<caption>`, `<thread>`, `<xref>`, and `<href>` within the element head.
- Add tests to validate the correct usage of element heads in various contexts.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="25280" yWindow="3480" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12680" yWindow="3960" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -524,23 +524,21 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Semantic elements capture core components with specific meaning and functional role in the document, for example, a paragraph, a table, a list, and more.
-Any semantic element may optionally begin with a [component head](#component-head-elements).
-Semantic elements are generally meant to be interpreted as block-level elements (although they can also be inlined via nesting).</t>
+          <t>*Semantic elements* capture core components with specific meaning and functional role in the document (e.g. a paragraph, a table, a list etc.) and may optionally begin with a [element head](#element-head).
+They are generally meant to be interpreted as block-level elements (although they can also be inlined via nesting).
+Semantic elements that can appear on the top level within `&lt;doclang&gt;` are called *primary*, while those that can only appear within other semantic elements are called *secondary*.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="85" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>component head</t>
+          <t>property</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>The component head is a sequence comprising the following elements in this order, whereby all elements are optional:&lt;br /&gt;&lt;ul&gt;&lt;li&gt;`&lt;thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;h_thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;xref&gt;` or `&lt;href&gt;` (mutually exclusive)&lt;/li&gt;&lt;li&gt;`&lt;meta&gt;`&lt;/li&gt;&lt;li&gt;sequence of 2*N `&lt;location&gt;`s (N&gt;1)&lt;/li&gt;&lt;li&gt;sequence of `&lt;timestamp&gt;`s&lt;/li&gt;&lt;li&gt;`&lt;layer&gt;`&lt;/li&gt;&lt;/ul&gt;
-A component head can only appear as the leading content of a semantic element.
-The various component head elements are further specified in the following subsections.</t>
+          <t>*Property elements* are non-semantic elements that help define useful traits of a semantic element, forming the main building blocks of the [element head](#element-head). Property elements that can appear on the top level of the element head are called *primary*, while those that can only appear within other property elements are called *secondary*. The various property elements are further specified in the following subsections.</t>
         </is>
       </c>
     </row>
@@ -603,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -612,8 +610,8 @@
     <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="10"/>
-    <col width="20" customWidth="1" style="1" min="11" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="11"/>
+    <col width="20" customWidth="1" style="1" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -644,7 +642,7 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>[Content] Component head</t>
+          <t>[Content] Element head</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -654,7 +652,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>[Content] Semantic elements</t>
+          <t>[Content] Primary semantic elements</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Is primary</t>
         </is>
       </c>
     </row>
@@ -793,6 +796,9 @@
       <c r="H5" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="I5" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -823,6 +829,9 @@
       <c r="H6" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="I6" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -832,7 +841,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>`&lt;caption&gt;`</t>
+          <t>`&lt;footnote&gt;`</t>
         </is>
       </c>
       <c r="C7" s="5" t="n"/>
@@ -853,6 +862,9 @@
       <c r="H7" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="I7" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -862,7 +874,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>`&lt;footnote&gt;`</t>
+          <t>`&lt;page_header&gt;`</t>
         </is>
       </c>
       <c r="C8" s="5" t="n"/>
@@ -883,6 +895,9 @@
       <c r="H8" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="I8" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -892,7 +907,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_header&gt;`</t>
+          <t>`&lt;page_footer&gt;`</t>
         </is>
       </c>
       <c r="C9" s="5" t="n"/>
@@ -913,6 +928,9 @@
       <c r="H9" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="I9" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -922,10 +940,14 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_footer&gt;`</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n"/>
+          <t>`&lt;field_region&gt;`</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Serves for scoping of field items, for example encapsulating a whole form.</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -938,13 +960,16 @@
         <v>1</v>
       </c>
       <c r="G10" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
+      <c r="I10" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="102" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>[01a] semantic (top)</t>
@@ -952,12 +977,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>`&lt;field_region&gt;`</t>
+          <t>`&lt;list&gt;`</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Serves for scoping of field items, for example encapsulating a whole form.</t>
+          <t>Captures a list. List items are delimited by the respective structural elements. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -968,17 +993,24 @@
       <c r="E11" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="F11" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" s="1" t="b">
-        <v>0</v>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, also on cell level in case of virtual `&lt;text&gt;` </t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+        </is>
       </c>
       <c r="H11" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" ht="102" customHeight="1">
+      <c r="I11" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="119" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>[01a] semantic (top)</t>
@@ -986,12 +1018,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>`&lt;list&gt;`</t>
+          <t>`&lt;table&gt;`</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Captures a list. List items are delimited by the respective structural elements. A list item can be defined without a wrapping tag, i.e. as pure (optional) component head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a table, in a format inspired by OTSL. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1015,8 +1047,11 @@
       <c r="H12" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" ht="119" customHeight="1">
+      <c r="I12" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>[01a] semantic (top)</t>
@@ -1024,14 +1059,10 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>`&lt;table&gt;`</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Captures a table, in a format inspired by OTSL. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) component head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
-        </is>
-      </c>
+          <t>`&lt;formula&gt;`</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1040,17 +1071,16 @@
       <c r="E13" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, also on cell level in case of virtual `&lt;text&gt;` </t>
-        </is>
-      </c>
-      <c r="G13" s="1" t="inlineStr">
-        <is>
-          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
-        </is>
+      <c r="F13" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="H13" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1062,7 +1092,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>`&lt;formula&gt;`</t>
+          <t>`&lt;code&gt;`</t>
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
@@ -1083,6 +1113,9 @@
       <c r="H14" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I14" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -1092,10 +1125,14 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>`&lt;code&gt;`</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n"/>
+          <t>`&lt;picture&gt;`</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Can contain specific semantic elements: `&lt;src&gt;`, `&lt;table&gt;`.</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1108,10 +1145,13 @@
         <v>1</v>
       </c>
       <c r="G15" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="I15" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
@@ -1122,7 +1162,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>`&lt;picture&gt;`</t>
+          <t>`&lt;marker&gt;`</t>
         </is>
       </c>
       <c r="C16" s="5" t="n"/>
@@ -1138,9 +1178,12 @@
         <v>1</v>
       </c>
       <c r="G16" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1152,10 +1195,14 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>`&lt;marker&gt;`</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n"/>
+          <t>`&lt;group&gt;`</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Container for encapsulating multiple semantic elements.</t>
+        </is>
+      </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1168,31 +1215,30 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>[01] semantic (top)</t>
+          <t>[01b] semantic (inner)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>`&lt;group&gt;`</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Container for encapsulating multiple semantic elements.</t>
-        </is>
-      </c>
+          <t>`&lt;field_heading&gt;`</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows semantic elements.</t>
+          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
         </is>
       </c>
       <c r="E18" s="6" t="b">
@@ -1202,10 +1248,13 @@
         <v>1</v>
       </c>
       <c r="G18" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="1" t="b">
         <v>1</v>
+      </c>
+      <c r="I18" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
@@ -1216,10 +1265,14 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>`&lt;field_heading&gt;`</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n"/>
+          <t>`&lt;field_item&gt;`</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Scoping of a field key (optional) and any corresponding values.</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Can only be descendant of `&lt;field_region&gt;`.</t>
@@ -1232,10 +1285,13 @@
         <v>1</v>
       </c>
       <c r="G19" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" s="1" t="b">
         <v>1</v>
+      </c>
+      <c r="I19" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="34" customHeight="1">
@@ -1246,17 +1302,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>`&lt;field_item&gt;`</t>
+          <t>`&lt;key&gt;`</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Scoping of a field key (optional) and any corresponding values.</t>
+          <t>The key of a field (may correspond to  0-N field values).</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
+          <t>Can only be descendant of `&lt;field_item&gt;`.</t>
         </is>
       </c>
       <c r="E20" s="6" t="b">
@@ -1266,10 +1322,13 @@
         <v>1</v>
       </c>
       <c r="G20" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" s="1" t="b">
         <v>1</v>
+      </c>
+      <c r="I20" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="34" customHeight="1">
@@ -1280,12 +1339,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>`&lt;key&gt;`</t>
+          <t>`&lt;value&gt;`</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>The key of a field (may correspond to  0-N field values).</t>
+          <t>A value of a field (may correspond to 0 or 1 field key).</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1304,6 +1363,9 @@
       </c>
       <c r="H21" s="1" t="b">
         <v>1</v>
+      </c>
+      <c r="I21" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1">
@@ -1314,17 +1376,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>`&lt;value&gt;`</t>
+          <t>`&lt;hint&gt;`</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>A value of a field (may correspond to 0 or 1 field key).</t>
+          <t>A hint regarding a field.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Can only be descendant of `&lt;field_item&gt;`.</t>
+          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
         </is>
       </c>
       <c r="E22" s="6" t="b">
@@ -1338,6 +1400,9 @@
       </c>
       <c r="H22" s="1" t="b">
         <v>1</v>
+      </c>
+      <c r="I22" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1">
@@ -1348,17 +1413,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>`&lt;hint&gt;`</t>
+          <t>`&lt;caption&gt;`</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>A hint regarding a field.</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
+          <t>Optional part of the element head for capturing an associated caption.</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Can only be part of the element head of a semantic element.</t>
         </is>
       </c>
       <c r="E23" s="6" t="b">
@@ -1372,12 +1437,15 @@
       </c>
       <c r="H23" s="1" t="b">
         <v>1</v>
+      </c>
+      <c r="I23" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="153" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1387,8 +1455,8 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the component head; serves for capturing a component spanning multiple bounding boxes (e.g. cross-column) or pages.&lt;br/&gt;
-To capture such a component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them.</t>
+          <t>Optional part of the element head; serves for establishing a logical document component. This can be useful for capturing fragmented components, e.g. spanning multiple bounding boxes (e.g. cross-column) or pages, or for defining anchors for cross references.&lt;br/&gt;
+To capture a fragmented component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1407,12 +1475,15 @@
       </c>
       <c r="H24" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I24" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25" ht="68" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1422,7 +1493,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the component head; serves for capturing a component crossing horizontal boundaries (e.g. table verically split between multiple pages).</t>
+          <t>Optional part of the element head; serves for capturing a component crossing horizontal boundaries (e.g. table verically split between multiple pages).</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1441,12 +1512,15 @@
       </c>
       <c r="H25" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I25" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26" ht="68" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1456,7 +1530,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the component head; serves for capturing an outgoing cross-reference from this component.</t>
+          <t>Optional part of the element head; serves for capturing an outgoing cross-reference from this component.</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1475,12 +1549,15 @@
       </c>
       <c r="H26" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I26" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1490,7 +1567,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the component head; serves for capturing a URI referenced by this component.</t>
+          <t>Optional part of the element head; serves for capturing a URI referenced by this component.</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -1509,12 +1586,15 @@
       </c>
       <c r="H27" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I27" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28" ht="34" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1543,12 +1623,15 @@
       </c>
       <c r="H28" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I28" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1577,12 +1660,15 @@
       </c>
       <c r="H29" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I29" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -1611,12 +1697,15 @@
       </c>
       <c r="H30" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I30" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31" ht="85" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1645,12 +1734,15 @@
       </c>
       <c r="H31" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I31" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1676,11 +1768,14 @@
       <c r="H32" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I32" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1706,11 +1801,14 @@
       <c r="H33" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I33" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1736,11 +1834,14 @@
       <c r="H34" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I34" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1766,11 +1867,14 @@
       <c r="H35" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I35" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>[03a] component head (outer)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1796,11 +1900,14 @@
       <c r="H36" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I36" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>[03b] component head (inner)</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1826,11 +1933,14 @@
       <c r="H37" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="I37" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>[03b] component head (inner)</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -1854,6 +1964,9 @@
         <v>1</v>
       </c>
       <c r="H38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor spec, separating out planned features
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12680" yWindow="3960" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12680" yWindow="3960" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -610,8 +610,8 @@
     <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="11"/>
-    <col width="20" customWidth="1" style="1" min="12" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="12"/>
+    <col width="20" customWidth="1" style="1" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -660,6 +660,11 @@
           <t>Is primary</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="51" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -708,7 +713,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Includes doc-level metadata. Also discussed in Appendix B.</t>
+          <t>Includes doc-level metadata.</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -1516,6 +1521,9 @@
       <c r="I25" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="J25" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26" ht="68" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -1738,6 +1746,9 @@
       <c r="I31" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="J31" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -1747,7 +1758,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>`&lt;hour&gt;`</t>
+          <t>`&lt;layer&gt;`</t>
         </is>
       </c>
       <c r="C32" s="5" t="n"/>
@@ -1775,12 +1786,12 @@
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>[03a] property (outer)</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>`&lt;minute&gt;`</t>
+          <t>`&lt;hour&gt;`</t>
         </is>
       </c>
       <c r="C33" s="5" t="n"/>
@@ -1802,18 +1813,21 @@
         <v>0</v>
       </c>
       <c r="I33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>[03a] property (outer)</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>`&lt;second&gt;`</t>
+          <t>`&lt;minute&gt;`</t>
         </is>
       </c>
       <c r="C34" s="5" t="n"/>
@@ -1835,18 +1849,21 @@
         <v>0</v>
       </c>
       <c r="I34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J34" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>[03a] property (outer)</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>`&lt;centisecond&gt;`</t>
+          <t>`&lt;second&gt;`</t>
         </is>
       </c>
       <c r="C35" s="5" t="n"/>
@@ -1868,18 +1885,21 @@
         <v>0</v>
       </c>
       <c r="I35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>[03a] property (outer)</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>`&lt;layer&gt;`</t>
+          <t>`&lt;centisecond&gt;`</t>
         </is>
       </c>
       <c r="C36" s="5" t="n"/>
@@ -1901,6 +1921,9 @@
         <v>0</v>
       </c>
       <c r="I36" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J36" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1936,6 +1959,9 @@
       <c r="I37" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="J37" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -1969,6 +1995,9 @@
       <c r="I38" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="J38" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39" ht="34" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
@@ -2627,7 +2656,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>New line / new table row</t>
+          <t>New line / new table row.</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -2725,6 +2754,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J61" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62" ht="17" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
@@ -2767,6 +2799,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J62" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="63" ht="17" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
@@ -2809,6 +2844,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J63" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64" ht="17" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
@@ -2823,33 +2861,25 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H64" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="65" ht="17" customHeight="1">
@@ -2893,6 +2923,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J65" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66" ht="17" customHeight="1">
       <c r="A66" s="7" t="inlineStr">
@@ -2935,6 +2968,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J66" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67" ht="17" customHeight="1">
       <c r="A67" s="7" t="inlineStr">
@@ -2977,6 +3013,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J67" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="68" ht="17" customHeight="1">
       <c r="A68" s="7" t="inlineStr">
@@ -3019,6 +3058,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J68" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69" ht="17" customHeight="1">
       <c r="A69" s="7" t="inlineStr">
@@ -3061,6 +3103,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J69" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="70" ht="17" customHeight="1">
       <c r="A70" s="7" t="inlineStr">
@@ -3103,6 +3148,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J70" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="71" ht="17" customHeight="1">
       <c r="A71" s="7" t="inlineStr">
@@ -3145,6 +3193,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J71" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="72" ht="17" customHeight="1">
       <c r="A72" s="7" t="inlineStr">
@@ -3187,6 +3238,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J72" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73" ht="17" customHeight="1">
       <c r="A73" s="7" t="inlineStr">
@@ -3229,6 +3283,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J73" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="74" ht="17" customHeight="1">
       <c r="A74" s="7" t="inlineStr">
@@ -3271,6 +3328,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J74" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="75" ht="17" customHeight="1">
       <c r="A75" s="7" t="inlineStr">
@@ -3313,6 +3373,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J75" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="76" ht="17" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
@@ -3355,6 +3418,9 @@
           <t>TBD</t>
         </is>
       </c>
+      <c r="J76" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77" ht="17" customHeight="1">
       <c r="A77" s="7" t="inlineStr">
@@ -3396,6 +3462,9 @@
         <is>
           <t>TBD</t>
         </is>
+      </c>
+      <c r="J77" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -3421,7 +3490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3515,51 +3584,61 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>`&lt;location&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>`value`</t>
+          <t>`width`</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; default "512"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Integer within [0, resolution)</t>
+          <t>Non-negative integer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Default document width in pixels.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>`&lt;location&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>`resolution`</t>
+          <t>`height`</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Optional; defaults to head metadata `&lt;default_resolution&gt;`, otherwise "512"</t>
+          <t>Optional; default "512"</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Positive integer</t>
+          <t>Non-negative integer</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Default document height in pixels.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>`&lt;hour&gt;`</t>
+          <t>`&lt;location&gt;`</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3574,36 +3653,36 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Non-negative integer</t>
+          <t>Integer within [0, resolution)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>`&lt;minute&gt;`</t>
+          <t>`&lt;location&gt;`</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>`value`</t>
+          <t>`resolution`</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; defaults to head metadata `&lt;default_resolution&gt;`, otherwise "512"</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Non-negative integer</t>
+          <t>Positive integer</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>`&lt;second&gt;`</t>
+          <t>`&lt;hour&gt;`</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3625,7 +3704,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>`&lt;centisecond&gt;`</t>
+          <t>`&lt;minute&gt;`</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3647,39 +3726,39 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>`&lt;layer&gt;`</t>
+          <t>`&lt;second&gt;`</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>`class`</t>
+          <t>`value`</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Optional; default: "body"</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>{"body", "furniture", "background", "invisible", "notes"}</t>
+          <t>Non-negative integer</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>`&lt;heading&gt;`</t>
+          <t>`&lt;centisecond&gt;`</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>`level`</t>
+          <t>`value`</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Optional; default "1"</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3691,7 +3770,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>`&lt;value&gt;`</t>
+          <t>`&lt;layer&gt;`</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3701,41 +3780,41 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Optional; default: "read_only"</t>
+          <t>Optional; default: "body"</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>{"read_only", "fillable"}</t>
+          <t>{"body", "furniture", "background", "invisible", "notes"}</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>`&lt;inline&gt;`</t>
+          <t>`&lt;heading&gt;`</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>`class`</t>
+          <t>`level`</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; default "1"</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>{"code", "formula", "picture"}</t>
+          <t>Non-negative integer</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>`&lt;list&gt;`</t>
+          <t>`&lt;value&gt;`</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3745,19 +3824,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Optional; default: "unordered"</t>
+          <t>Optional; default: "read_only"</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>{"unordered", "ordered"}</t>
+          <t>{"read_only", "fillable"}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>`&lt;table&gt;`</t>
+          <t>`&lt;inline&gt;`</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3767,24 +3846,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Optional; default: "data"</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>{"data", "index"}</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>A value of "index" denotes a document index as it would be used e.g. for a table of contents.</t>
+          <t>{"code", "formula", "picture"}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>`&lt;floating_group&gt;`</t>
+          <t>`&lt;list&gt;`</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3794,19 +3868,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; default: "unordered"</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"table", "picture", "code", "formula"}</t>
+          <t>{"unordered", "ordered"}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
+          <t>`&lt;table&gt;`</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3816,24 +3890,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Optional; default: "unselected"</t>
+          <t>Optional; default: "data"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>{"unselected", "selected"}</t>
+          <t>{"data", "index"}</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>A value of "index" denotes a document index as it would be used e.g. for a table of contents.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>`&lt;thread&gt;`</t>
+          <t>`&lt;floating_group&gt;`</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>`thread_id`</t>
+          <t>`class`</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3843,41 +3922,36 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Positive integer</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>A string that identifies a thread.</t>
+          <t>{"table", "picture", "code", "formula"}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>`&lt;h_thread&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>`h_thread_id`</t>
+          <t>`class`</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; default: "unselected"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Positive integer</t>
+          <t>{"unselected", "selected"}</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>`&lt;xref&gt;`</t>
+          <t>`&lt;thread&gt;`</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3897,19 +3971,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>The ID of the referenced thread.</t>
+          <t>A string that identifies a thread.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>`&lt;href&gt;`</t>
+          <t>`&lt;h_thread&gt;`</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>`uri`</t>
+          <t>`h_thread_id`</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3919,44 +3993,100 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>URI</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>The URI of the referenced resource.</t>
+          <t>Positive integer</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>`&lt;xref&gt;`</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>`thread_id`</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>The ID of the referenced thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>`&lt;href&gt;`</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>`uri`</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>The URI of the referenced resource.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>`&lt;src&gt;`</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>`uri`</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>URI</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>The source URI.</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>`</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
add `<default_resolution>` to validator, add tests, align `<h_thread>`
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -610,8 +610,8 @@
     <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="12"/>
-    <col width="20" customWidth="1" style="1" min="13" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="13"/>
+    <col width="20" customWidth="1" style="1" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1780,6 +1780,9 @@
         <v>0</v>
       </c>
       <c r="I32" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3490,7 +3493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4078,13 +4081,6 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>`</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:E12"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add `<custom>`, defer `<meta>`
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -610,8 +610,8 @@
     <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="13"/>
-    <col width="20" customWidth="1" style="1" min="14" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="14"/>
+    <col width="20" customWidth="1" style="1" min="15" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1635,6 +1635,9 @@
       <c r="I28" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="J28" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -1644,7 +1647,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>`&lt;custom_meta&gt;`</t>
+          <t>`&lt;custom&gt;`</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -3493,7 +3496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3910,7 +3913,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>`&lt;floating_group&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3920,46 +3923,51 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; default: "unselected"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>{"table", "picture", "code", "formula"}</t>
+          <t>{"unselected", "selected"}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
+          <t>`&lt;thread&gt;`</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>`class`</t>
+          <t>`thread_id`</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Optional; default: "unselected"</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>{"unselected", "selected"}</t>
+          <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A string that identifies a thread.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>`&lt;thread&gt;`</t>
+          <t>`&lt;h_thread&gt;`</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>`thread_id`</t>
+          <t>`h_thread_id`</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3970,23 +3978,18 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>Positive integer</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>A string that identifies a thread.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>`&lt;h_thread&gt;`</t>
+          <t>`&lt;xref&gt;`</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>`h_thread_id`</t>
+          <t>`thread_id`</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3997,18 +4000,23 @@
       <c r="D21" t="inlineStr">
         <is>
           <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>The ID of the referenced thread.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>`&lt;xref&gt;`</t>
+          <t>`&lt;href&gt;`</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>`thread_id`</t>
+          <t>`uri`</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4018,19 +4026,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Positive integer</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>The ID of the referenced thread.</t>
+          <t>The URI of the referenced resource.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>`&lt;href&gt;`</t>
+          <t>`&lt;src&gt;`</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4049,33 +4057,6 @@
         </is>
       </c>
       <c r="E23" t="inlineStr">
-        <is>
-          <t>The URI of the referenced resource.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>`&lt;src&gt;`</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>`uri`</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>URI</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
         <is>
           <t>The source URI.</t>
         </is>

</xml_diff>

<commit_message>
enhance `location@value` validation in schema and documentation
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -610,8 +610,8 @@
     <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="15"/>
-    <col width="20" customWidth="1" style="1" min="16" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="16"/>
+    <col width="20" customWidth="1" style="1" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3649,17 +3649,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>`value`</t>
+          <t>`resolution`</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; defaults to `default_resolution@width` or `default_resolution@height` depending on whether location refers to x or y, otherwise "512" if respective `default_resolution` not explicitly specified</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Integer within [0, resolution)</t>
+          <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Axis boundary (exclusive) for the respective `location@value`.</t>
         </is>
       </c>
     </row>
@@ -3671,17 +3676,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>`resolution`</t>
+          <t>`value`</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Optional; defaults to head metadata `&lt;default_resolution&gt;`, otherwise "512"</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Positive integer</t>
+          <t>Integer within [0, `location.resolution`)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor spec for clarity and correctness
- Removed outdated TODO comments regarding table continuation.
- Updated cross-reference example to clarify inline usage.
- Revised page break handling instructions for consistency.
- Adjusted definitions for `<nl>` and `<thread>` elements to enhance understanding.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12680" yWindow="3960" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12680" yWindow="3960" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -697,7 +697,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>New line / new table row.</t>
+          <t>Denotes the end of a table row.</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">

</xml_diff>

<commit_message>
add `<label>`, document recommended values
- Introduced `<label>` element for subclassing core components and improved extensibility.
- Updated element head definitions to include `<label>` as a property element.
- Revised validation rules in the schema to accommodate the new `<label>` element.
- Added examples demonstrating the use of `<label>` in various contexts, including `<code>` and `<picture>` elements.
- Removed deprecated `<br>` element from the schema and updated related tests.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12680" yWindow="3960" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -601,17 +601,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
     <col width="28.5" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
     <col width="40.5" customWidth="1" style="2" min="3" max="3"/>
-    <col width="34.83203125" customWidth="1" style="2" min="4" max="4"/>
+    <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="16"/>
-    <col width="20" customWidth="1" style="1" min="17" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="17"/>
+    <col width="20" customWidth="1" style="1" min="18" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1028,62 +1028,70 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Captures a table, in a format inspired by OTSL. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a table in an OTSL-based format. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
+          <t>Any context that allows semantic elements. And additionally as the first element of the element body of `&lt;picture class="chart"&gt;`.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, also on cell level in case of virtual `&lt;text&gt;` </t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="119" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>[01a] semantic (top)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;index&gt;`</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Cells are delimited by the respective structural elements. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
           <t>Any context that allows semantic elements.</t>
         </is>
       </c>
-      <c r="E12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="E13" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE, also on cell level in case of virtual `&lt;text&gt;` </t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
         </is>
       </c>
-      <c r="H12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>[01a] semantic (top)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;formula&gt;`</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Any context that allows semantic elements.</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="H13" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="1" t="b">
         <v>1</v>
@@ -1097,7 +1105,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>`&lt;code&gt;`</t>
+          <t>`&lt;formula&gt;`</t>
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
@@ -1130,14 +1138,10 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>`&lt;picture&gt;`</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Can contain specific semantic elements: `&lt;src&gt;`, `&lt;table&gt;`.</t>
-        </is>
-      </c>
+          <t>`&lt;code&gt;`</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1150,10 +1154,10 @@
         <v>1</v>
       </c>
       <c r="G15" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="1" t="b">
         <v>1</v>
@@ -1167,10 +1171,14 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>`&lt;marker&gt;`</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n"/>
+          <t>`&lt;picture&gt;`</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Can contain a `&lt;src&gt;`. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;` or with a `&lt;smiles&gt;` in case of `&lt;picture class="chemistry"&gt;`.</t>
+        </is>
+      </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1183,7 +1191,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" s="1" t="b">
         <v>1</v>
@@ -1200,14 +1208,10 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>`&lt;group&gt;`</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Container for encapsulating multiple semantic elements.</t>
-        </is>
-      </c>
+          <t>`&lt;marker&gt;`</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n"/>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1220,7 +1224,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="1" t="b">
         <v>1</v>
@@ -1232,18 +1236,22 @@
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>[01b] semantic (inner)</t>
+          <t>[01a] semantic (top)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>`&lt;field_heading&gt;`</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n"/>
+          <t>`&lt;group&gt;`</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Container for encapsulating multiple semantic elements.</t>
+        </is>
+      </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
+          <t>Any context that allows semantic elements.</t>
         </is>
       </c>
       <c r="E18" s="6" t="b">
@@ -1253,13 +1261,13 @@
         <v>1</v>
       </c>
       <c r="G18" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" s="1" t="b">
         <v>1</v>
       </c>
       <c r="I18" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
@@ -1270,14 +1278,10 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>`&lt;field_item&gt;`</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Scoping of a field key (optional) and any corresponding values.</t>
-        </is>
-      </c>
+          <t>`&lt;field_heading&gt;`</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n"/>
       <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Can only be descendant of `&lt;field_region&gt;`.</t>
@@ -1290,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="1" t="b">
         <v>1</v>
@@ -1307,17 +1311,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>`&lt;key&gt;`</t>
+          <t>`&lt;field_item&gt;`</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>The key of a field (may correspond to  0-N field values).</t>
+          <t>Scoping of a field key (optional) and any corresponding values.</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Can only be descendant of `&lt;field_item&gt;`.</t>
+          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
         </is>
       </c>
       <c r="E20" s="6" t="b">
@@ -1327,7 +1331,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="1" t="b">
         <v>1</v>
@@ -1344,12 +1348,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>`&lt;value&gt;`</t>
+          <t>`&lt;key&gt;`</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>A value of a field (may correspond to 0 or 1 field key).</t>
+          <t>The key of a field (may correspond to  0-N field values).</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1381,17 +1385,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>`&lt;hint&gt;`</t>
+          <t>`&lt;value&gt;`</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>A hint regarding a field.</t>
+          <t>A value of a field (may correspond to 0 or 1 field key).</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
+          <t>Can only be descendant of `&lt;field_item&gt;`.</t>
         </is>
       </c>
       <c r="E22" s="6" t="b">
@@ -1418,210 +1422,210 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
+          <t>`&lt;hint&gt;`</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>A hint regarding a field.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Can only be descendant of `&lt;field_region&gt;`.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>[01b] semantic (inner)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
           <t>`&lt;caption&gt;`</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Optional part of the element head for capturing an associated caption.</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Can only be part of the element head of a semantic element.</t>
         </is>
       </c>
-      <c r="E23" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F23" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G23" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="153" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="E24" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="153" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;label&gt;`</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Optional part of the element head; serves for providing a detailed label for the respective element.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" ht="153" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>`&lt;thread&gt;`</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Optional part of the element head; serves for establishing a logical document component. This can be useful for capturing fragmented components, e.g. spanning multiple bounding boxes (e.g. cross-column) or pages, or for defining anchors for cross references.&lt;br/&gt;
 To capture a fragmented component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
         </is>
       </c>
-      <c r="E24" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G24" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I24" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" ht="68" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="E26" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" ht="68" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>`&lt;h_thread&gt;`</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Optional part of the element head; serves for capturing a component crossing horizontal boundaries (e.g. table verically split between multiple pages).</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
         </is>
       </c>
-      <c r="E25" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F25" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G25" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H25" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I25" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J25" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" ht="68" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="E27" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G27" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" ht="68" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>`&lt;xref&gt;`</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Optional part of the element head; serves for capturing an outgoing cross-reference from this component.</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element. Mutually exclusive with `&lt;href&gt;`.</t>
         </is>
       </c>
-      <c r="E26" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F26" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H26" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I26" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>[03a] property (outer)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;href&gt;`</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Optional part of the element head; serves for capturing a URI referenced by this component.</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;xref&gt;`.</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F27" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G27" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H27" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I27" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>[03a] property (outer)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;meta&gt;`</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Used to store additional or derived information regarding the respective component.</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
       <c r="E28" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" s="6" t="b">
         <v>0</v>
@@ -1633,9 +1637,6 @@
         <v>0</v>
       </c>
       <c r="I28" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J28" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1647,17 +1648,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>`&lt;custom&gt;`</t>
+          <t>`&lt;href&gt;`</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Custom metadata, e.g. for application-specific purposes.</t>
+          <t>Optional part of the element head; serves for capturing a URI referenced by this component.</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;xref&gt;`.</t>
         </is>
       </c>
       <c r="E29" s="6" t="b">
@@ -1667,7 +1668,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29" s="1" t="b">
         <v>0</v>
@@ -1682,132 +1683,137 @@
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;meta&gt;`</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Used to store additional or derived information regarding the respective component.</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F30" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;custom&gt;`</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Custom metadata, e.g. for application-specific purposes.</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F31" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G31" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H31" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>`&lt;location&gt;`</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Coordinate system is the bottom-left corner of the page.</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
         </is>
       </c>
-      <c r="E30" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F30" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G30" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H30" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I30" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" ht="85" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="E32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" ht="85" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>`&lt;timestamp&gt;`</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>TBD. Needed, if the individual hour/minute/etc are not all required (else cannot unambiguously interpret `&lt;hour&gt;0&lt;/hour&gt;&lt;minute&gt;2&lt;/minute&gt;&lt;second&gt;3&lt;/second&gt;`)</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
         </is>
       </c>
-      <c r="E31" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F31" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G31" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H31" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I31" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J31" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" ht="17" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>[03a] property (outer)</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;layer&gt;`</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I32" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J32" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>[03b] property (inner)</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;hour&gt;`</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
       <c r="E33" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="6" t="b">
         <v>0</v>
@@ -1819,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" s="1" t="b">
         <v>1</v>
@@ -1828,12 +1834,12 @@
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>[03b] property (inner)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>`&lt;minute&gt;`</t>
+          <t>`&lt;layer&gt;`</t>
         </is>
       </c>
       <c r="C34" s="5" t="n"/>
@@ -1855,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" s="1" t="b">
         <v>1</v>
@@ -1869,7 +1875,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>`&lt;second&gt;`</t>
+          <t>`&lt;hour&gt;`</t>
         </is>
       </c>
       <c r="C35" s="5" t="n"/>
@@ -1905,7 +1911,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>`&lt;centisecond&gt;`</t>
+          <t>`&lt;minute&gt;`</t>
         </is>
       </c>
       <c r="C36" s="5" t="n"/>
@@ -1941,23 +1947,23 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;second&gt;`</t>
         </is>
       </c>
       <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;meta&gt;`.</t>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
         </is>
       </c>
       <c r="E37" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G37" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H37" s="1" t="b">
         <v>0</v>
@@ -1977,99 +1983,107 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>`&lt;classification&gt;`</t>
+          <t>`&lt;centisecond&gt;`</t>
         </is>
       </c>
       <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F38" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J38" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>[03b] property (inner)</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;summary&gt;`</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;meta&gt;`.</t>
         </is>
       </c>
-      <c r="E38" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F38" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G38" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H38" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I38" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J38" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" ht="34" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>[04] payload</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;src&gt;`</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>The image's source.</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;picture&gt;`.</t>
-        </is>
-      </c>
       <c r="E39" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G39" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="I39" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J39" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="17" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>[04] payload</t>
+          <t>[03b] property (inner)</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
+          <t>`&lt;classification&gt;`</t>
         </is>
       </c>
       <c r="C40" s="5" t="n"/>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be child of `&lt;meta&gt;`.</t>
         </is>
       </c>
       <c r="E40" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G40" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" ht="17" customHeight="1">
+      <c r="I40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J40" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" ht="34" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
@@ -2077,23 +2091,27 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>`&lt;content&gt;`</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="n"/>
+          <t>`&lt;src&gt;`</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>The image's source.</t>
+        </is>
+      </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be child of `&lt;picture&gt;`.</t>
         </is>
       </c>
       <c r="E41" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G41" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41" s="1" t="b">
         <v>0</v>
@@ -2102,12 +2120,12 @@
     <row r="42" ht="17" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="C42" s="5" t="n"/>
@@ -2117,13 +2135,13 @@
         </is>
       </c>
       <c r="E42" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G42" s="6" t="b">
-        <v>1</v>
+      <c r="G42" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H42" s="1" t="b">
         <v>0</v>
@@ -2132,12 +2150,12 @@
     <row r="43" ht="17" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
+          <t>`&lt;content&gt;`</t>
         </is>
       </c>
       <c r="C43" s="5" t="n"/>
@@ -2152,7 +2170,7 @@
       <c r="F43" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G43" s="6" t="b">
+      <c r="G43" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H43" s="1" t="b">
@@ -2162,27 +2180,31 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="n"/>
+          <t>`&lt;smiles&gt;`</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>The SMILES representation of a molecule.</t>
+        </is>
+      </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be the first element of the element body of `&lt;picture class="chemistry"&gt;`.</t>
         </is>
       </c>
       <c r="E44" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G44" s="6" t="b">
+      <c r="G44" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="b">
@@ -2197,7 +2219,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
+          <t>`&lt;bold&gt;`</t>
         </is>
       </c>
       <c r="C45" s="5" t="n"/>
@@ -2227,7 +2249,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
+          <t>`&lt;italic&gt;`</t>
         </is>
       </c>
       <c r="C46" s="5" t="n"/>
@@ -2257,7 +2279,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
+          <t>`&lt;underline&gt;`</t>
         </is>
       </c>
       <c r="C47" s="5" t="n"/>
@@ -2287,7 +2309,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
+          <t>`&lt;strikethrough&gt;`</t>
         </is>
       </c>
       <c r="C48" s="5" t="n"/>
@@ -2317,14 +2339,10 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Indicates right-to-left direction.</t>
-        </is>
-      </c>
+          <t>`&lt;superscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="n"/>
       <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2346,32 +2364,28 @@
     <row r="50" ht="17" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
-        </is>
-      </c>
+          <t>`&lt;subscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n"/>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E50" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G50" s="1" t="b">
-        <v>0</v>
+      <c r="G50" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H50" s="1" t="b">
         <v>0</v>
@@ -2380,32 +2394,28 @@
     <row r="51" ht="17" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Indicates the beginning of an empty cell.</t>
-        </is>
-      </c>
+          <t>`&lt;handwriting&gt;`</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n"/>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E51" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F51" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G51" s="1" t="b">
-        <v>0</v>
+      <c r="G51" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H51" s="1" t="b">
         <v>0</v>
@@ -2414,32 +2424,32 @@
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;rtl&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates right-to-left direction.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E52" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F52" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G52" s="1" t="b">
-        <v>0</v>
+      <c r="G52" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H52" s="1" t="b">
         <v>0</v>
@@ -2453,17 +2463,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rhed&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a row header cell.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E53" s="6" t="b">
@@ -2479,7 +2489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" ht="34" customHeight="1">
+    <row r="54" ht="17" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2487,17 +2497,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;corn&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E54" s="6" t="b">
@@ -2521,17 +2531,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>`&lt;srow&gt;`</t>
+          <t>`&lt;ched&gt;`</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a section row header.</t>
+          <t>Indicates the beginning of a column header cell.</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E55" s="6" t="b">
@@ -2547,7 +2557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" ht="51" customHeight="1">
+    <row r="56" ht="17" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2555,17 +2565,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>`&lt;lcel&gt;`</t>
+          <t>`&lt;rhed&gt;`</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+          <t>Indicates the beginning of a row header cell.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E56" s="6" t="b">
@@ -2589,17 +2599,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ucel&gt;`</t>
+          <t>`&lt;corn&gt;`</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E57" s="6" t="b">
@@ -2615,7 +2625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" ht="51" customHeight="1">
+    <row r="58" ht="17" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2623,17 +2633,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>`&lt;xcel&gt;`</t>
+          <t>`&lt;srow&gt;`</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
+          <t>Indicates the beginning of a section row header.</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E58" s="6" t="b">
@@ -2649,7 +2659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="17" customHeight="1">
+    <row r="59" ht="51" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2657,17 +2667,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>`&lt;nl&gt;`</t>
+          <t>`&lt;lcel&gt;`</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Denotes the end of a table row.</t>
+          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E59" s="6" t="b">
@@ -2691,21 +2701,21 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ldiv&gt;`</t>
+          <t>`&lt;ucel&gt;`</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
+          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;list&gt;`.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E60" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F60" s="6" t="b">
         <v>0</v>
@@ -2713,145 +2723,112 @@
       <c r="G60" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H60" s="1" t="inlineStr">
-        <is>
-          <t>Only `&lt;marker&gt;`</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="17" customHeight="1">
+      <c r="H60" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" ht="51" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>`&lt;title&gt;`</t>
-        </is>
-      </c>
-      <c r="C61" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D61" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G61" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J61" s="1" t="b">
-        <v>1</v>
+          <t>`&lt;xcel&gt;`</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="62" ht="17" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J62" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" ht="17" customHeight="1">
+          <t>`&lt;nl&gt;`</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Denotes the end of a table row.</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H62" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="34" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J63" s="1" t="b">
-        <v>1</v>
+          <t>`&lt;ldiv&gt;`</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;list&gt;`.</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F63" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G63" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>Only `&lt;marker&gt;`</t>
+        </is>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
@@ -2862,30 +2839,41 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;title&gt;`</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F64" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G64" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H64" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J64" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="65" ht="17" customHeight="1">
@@ -2896,7 +2884,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2941,7 +2929,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -2986,41 +2974,30 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J67" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H67" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3031,7 +3008,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3076,7 +3053,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -3121,7 +3098,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3166,7 +3143,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3211,7 +3188,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3256,7 +3233,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3301,7 +3278,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3346,7 +3323,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3391,7 +3368,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3436,55 +3413,190 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
+          <t>`&lt;stewardship&gt;`</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J77" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" ht="17" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;access_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J78" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" ht="17" customHeight="1">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;retention_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J79" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" ht="17" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
           <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G77" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J77" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="1" t="n"/>
-      <c r="B78" s="1" t="n"/>
-      <c r="C78" s="1" t="n"/>
-      <c r="D78" s="1" t="n"/>
-      <c r="F78" s="1" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="n"/>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n"/>
+      <c r="B81" s="1" t="n"/>
+      <c r="C81" s="1" t="n"/>
+      <c r="D81" s="1" t="n"/>
+      <c r="F81" s="1" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H77"/>
+  <autoFilter ref="A1:H80"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3847,7 +3959,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>`&lt;inline&gt;`</t>
+          <t>`&lt;list&gt;`</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3857,19 +3969,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional; default: "unordered"</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>{"code", "formula", "picture"}</t>
+          <t>{"unordered", "ordered"}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>`&lt;list&gt;`</t>
+          <t>`&lt;picture&gt;`</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3879,19 +3991,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Optional; default: "unordered"</t>
+          <t>Optional; default: "unspecified"</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"unordered", "ordered"}</t>
+          <t>{"unspecified", "chart", "chemistry"}</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>The picture type.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>`&lt;table&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3901,39 +4018,39 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Optional; default: "data"</t>
+          <t>Optional; default: "unselected"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>{"data", "index"}</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>A value of "index" denotes a document index as it would be used e.g. for a table of contents.</t>
+          <t>{"unselected", "selected"}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
+          <t>`&lt;label&gt;`</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>`class`</t>
+          <t>`value`</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Optional; default: "unselected"</t>
+          <t>Optional; default: "unspecified"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>{"unselected", "selected"}</t>
+          <t>Different value domains may be recommended per host element (not to be validated).</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>A label for concretely specifying a subclass type for the host element.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
improve documentation of `<formula>`, `<superscript>` & `<subscript>`
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="17"/>
-    <col width="20" customWidth="1" style="1" min="18" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="18"/>
+    <col width="20" customWidth="1" style="1" min="19" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1108,7 +1108,11 @@
           <t>`&lt;formula&gt;`</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n"/>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Raw LaTeX formula content, i.e. without any LaTeX-specific wrapping such as `$ ... $`, `$$ ... $$`,  `\( ... \)`, `\[ ... \]`, `\begin{math} ... \end{math}` or `\begin{equation} ... \end{equation}`.</t>
+        </is>
+      </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>

</xml_diff>

<commit_message>
clarify `<picture>`/`<src>`, update default class/label & picture labels
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="18"/>
-    <col width="20" customWidth="1" style="1" min="19" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="19"/>
+    <col width="20" customWidth="1" style="1" min="20" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Can contain a `&lt;src&gt;`. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;` or with a `&lt;smiles&gt;` in case of `&lt;picture class="chemistry"&gt;`.</t>
+          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;` or with a `&lt;smiles&gt;` in case of `&lt;picture class="chemistry"&gt;`.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -3995,12 +3995,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Optional; default: "unspecified"</t>
+          <t>Optional; default: "undefined"</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"unspecified", "chart", "chemistry"}</t>
+          <t>{"undefined", "chart", "chemistry"}</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Optional; default: "unspecified"</t>
+          <t>Optional; default: "undefined"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>The source URI.</t>
+          <t>The source URI. May use a `data:` URI (RFC 2397) with base64-encoded payload, e.g. `uri="data:image/png;base64,…"`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
extend `<picture>` documentation, detail `src.uri`, improve `<smiles>`
- Clarified subclassing of core document components using the `<label>` element.
- Added detailed examples for `<picture>` usage, including image sourcing via URI and base64 encoding.
- Updated the `<smiles>` element in the schema to allow mixed content.
- Revised existing test cases to reflect changes in `<picture>` and `<smiles>` usage.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="19"/>
-    <col width="20" customWidth="1" style="1" min="20" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="20"/>
+    <col width="20" customWidth="1" style="1" min="21" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -2203,7 +2203,7 @@
         </is>
       </c>
       <c r="E44" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44" s="6" t="b">
         <v>0</v>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>The source URI. May use a `data:` URI (RFC 2397) with base64-encoded payload, e.g. `uri="data:image/png;base64,…"`.</t>
+          <t>The source URI. May use a `data:` URI (RFC 2397) with base64-encoded payload, e.g. `uri="data:image/png;base64,…"`. Relative URIs are allowed too, e.g. `uri="assets/chart.svg"`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refine `<picture>` subclassing, update examples
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="20"/>
-    <col width="20" customWidth="1" style="1" min="21" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="21"/>
+    <col width="20" customWidth="1" style="1" min="22" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;` or with a `&lt;smiles&gt;` in case of `&lt;picture class="chemistry"&gt;`.</t>
+          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2184,22 +2184,18 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>[04] payload</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>`&lt;smiles&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>The SMILES representation of a molecule.</t>
-        </is>
-      </c>
+          <t>`&lt;bold&gt;`</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n"/>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Can only be the first element of the element body of `&lt;picture class="chemistry"&gt;`.</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E44" s="6" t="b">
@@ -2208,7 +2204,7 @@
       <c r="F44" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G44" s="1" t="b">
+      <c r="G44" s="6" t="b">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="b">
@@ -2223,7 +2219,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
+          <t>`&lt;italic&gt;`</t>
         </is>
       </c>
       <c r="C45" s="5" t="n"/>
@@ -2253,7 +2249,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
+          <t>`&lt;underline&gt;`</t>
         </is>
       </c>
       <c r="C46" s="5" t="n"/>
@@ -2283,7 +2279,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
+          <t>`&lt;strikethrough&gt;`</t>
         </is>
       </c>
       <c r="C47" s="5" t="n"/>
@@ -2313,7 +2309,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
+          <t>`&lt;superscript&gt;`</t>
         </is>
       </c>
       <c r="C48" s="5" t="n"/>
@@ -2343,7 +2339,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
+          <t>`&lt;subscript&gt;`</t>
         </is>
       </c>
       <c r="C49" s="5" t="n"/>
@@ -2373,7 +2369,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
+          <t>`&lt;handwriting&gt;`</t>
         </is>
       </c>
       <c r="C50" s="5" t="n"/>
@@ -2403,10 +2399,14 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="n"/>
+          <t>`&lt;rtl&gt;`</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Indicates right-to-left direction.</t>
+        </is>
+      </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2428,32 +2428,32 @@
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates right-to-left direction.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E52" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G52" s="6" t="b">
-        <v>1</v>
+      <c r="G52" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H52" s="1" t="b">
         <v>0</v>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;ched&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates the beginning of a column header cell.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -2535,12 +2535,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;rhed&gt;`</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of a row header cell.</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2561,7 +2561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" ht="17" customHeight="1">
+    <row r="56" ht="34" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2569,12 +2569,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rhed&gt;`</t>
+          <t>`&lt;corn&gt;`</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a row header cell.</t>
+          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2595,7 +2595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" ht="34" customHeight="1">
+    <row r="57" ht="17" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2603,12 +2603,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>`&lt;corn&gt;`</t>
+          <t>`&lt;srow&gt;`</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+          <t>Indicates the beginning of a section row header.</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2629,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" ht="17" customHeight="1">
+    <row r="58" ht="51" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2637,12 +2637,12 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>`&lt;srow&gt;`</t>
+          <t>`&lt;lcel&gt;`</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a section row header.</t>
+          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -2663,7 +2663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="51" customHeight="1">
+    <row r="59" ht="34" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2671,12 +2671,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>`&lt;lcel&gt;`</t>
+          <t>`&lt;ucel&gt;`</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -2697,7 +2697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" ht="34" customHeight="1">
+    <row r="60" ht="51" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2705,12 +2705,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ucel&gt;`</t>
+          <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" ht="51" customHeight="1">
+    <row r="61" ht="17" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2739,12 +2739,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>`&lt;xcel&gt;`</t>
+          <t>`&lt;nl&gt;`</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
+          <t>Denotes the end of a table row.</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -2765,7 +2765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" ht="17" customHeight="1">
+    <row r="62" ht="34" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2773,21 +2773,21 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>`&lt;nl&gt;`</t>
+          <t>`&lt;ldiv&gt;`</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Denotes the end of a table row.</t>
+          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Can only be child of `&lt;list&gt;`.</t>
         </is>
       </c>
       <c r="E62" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F62" s="6" t="b">
         <v>0</v>
@@ -2795,44 +2795,55 @@
       <c r="G62" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H62" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" ht="34" customHeight="1">
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>Only `&lt;marker&gt;`</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="17" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[07] document head</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ldiv&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;list&gt;`.</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F63" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G63" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H63" s="1" t="inlineStr">
-        <is>
-          <t>Only `&lt;marker&gt;`</t>
-        </is>
+          <t>`&lt;title&gt;`</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
@@ -2843,7 +2854,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;title&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2888,7 +2899,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2933,41 +2944,30 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J66" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F66" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G66" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H66" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="67" ht="17" customHeight="1">
@@ -2978,30 +2978,41 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H67" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J67" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3012,7 +3023,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3057,7 +3068,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -3102,7 +3113,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3147,7 +3158,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3192,7 +3203,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3237,7 +3248,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3282,7 +3293,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3327,7 +3338,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3372,7 +3383,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3417,7 +3428,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;access_policy&gt;`</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3462,7 +3473,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;retention_policy&gt;`</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -3507,7 +3518,7 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -3544,63 +3555,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" ht="17" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>[07] document head</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;compliance_requirements&gt;`</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="b">
-        <v>1</v>
-      </c>
+    <row r="80">
+      <c r="A80" s="1" t="n"/>
+      <c r="B80" s="1" t="n"/>
+      <c r="C80" s="1" t="n"/>
+      <c r="D80" s="1" t="n"/>
+      <c r="F80" s="1" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n"/>
-      <c r="B81" s="1" t="n"/>
-      <c r="C81" s="1" t="n"/>
-      <c r="D81" s="1" t="n"/>
-      <c r="F81" s="1" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="n"/>
+      <c r="A81" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H80"/>
+  <autoFilter ref="A1:H79"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -4000,7 +3966,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"undefined", "chart", "chemistry"}</t>
+          <t>{"undefined", "chart"}</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">

</xml_diff>

<commit_message>
improve `<location>` handling, various spec refinements
- Tightened location rules: exactly 4 coords (`x_min,y_min,x_max,y_max`) with normalized order checks and new valid/invalid fixtures.
- Cleaned up `spec.md`: clarified structural constraints, reorganized appendices, and aligned terminology.
- Extended `<marker>` to support element-head metadata (including location) in XSD/Schematron, plus coverage tests.
- Improved DOCX export TOC/heading pagination flow and regenerated reference `.docx`/`.xlsx` outputs.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="21"/>
-    <col width="20" customWidth="1" style="1" min="22" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="23"/>
+    <col width="20" customWidth="1" style="1" min="24" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -987,7 +987,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Captures a list. List items are delimited by the respective structural elements. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a list. List items are started by the respective structural elements (`&lt;ldiv&gt;`). A non-empty `&lt;list&gt;` element body must begin with such a structural element. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Captures a table in an OTSL-based format. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a table in an OTSL-based format. Table cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;table&gt;` element body must begin with such a structural element. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Cells are delimited by the respective structural elements. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Index cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;index&gt;` element body must begin with such a structural element. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`.</t>
+          <t>Element body can generally only contain a `&lt;src&gt;`, for image bytes or reference. Additionally, in case of `&lt;picture class="chart"&gt;` (and only then) the element body may contain a `&lt;table&gt;`, in which case it must begin with it.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1197,8 +1197,10 @@
       <c r="G16" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="1" t="b">
-        <v>1</v>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Not allowed (except `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`)</t>
+        </is>
       </c>
       <c r="I16" s="1" t="b">
         <v>1</v>
@@ -1694,7 +1696,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Used to store additional or derived information regarding the respective component.</t>
+          <t>Optional part of the element head; used to store additional or derived information regarding the respective component.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1734,7 +1736,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Custom metadata, e.g. for application-specific purposes.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1771,7 +1773,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Coordinate system is the bottom-left corner of the page.</t>
+          <t>Optional part of the element head; coordinate system is the top-left corner of the page. When present, appears in sequence of 4 `&lt;location&gt;` instances, representing x0, y0, x1, y1. The following must then hold: `x0_norm&lt;=x1_norm` and `y0_norm&lt;=y1_norm`(i.e. first top-left point then bottom-right point), whereby `*_norm` is the respective coordinate normalized to its effective resolution.</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3771,6 +3773,11 @@
           <t>Integer within [0, `location.resolution`)</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Coordinate w.r.t. top-left corner.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4047,7 +4054,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A string that identifies a thread.</t>
+          <t>The ID of the thread. All `&lt;thread&gt;` elements that share a given `thread_id` must be under the same host element type (e.g. all under `&lt;text&gt;`, not mixed `&lt;text&gt;` and `&lt;picture&gt;`).</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4103,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>The ID of the referenced thread.</t>
+          <t>The ID of the referenced thread. This must be defined by at least one `&lt;thread&gt;` in the document.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
enforce field scope rules, expand recommendation guidance
- Add Schematron rules to enforce field placement (`field_heading`/`field_item` under `field_region`, `key`/`value` under `field_item`) and own-key cardinality per `field_item`.
- Update valid/invalid XML fixtures to cover misplaced elements, duplicate own keys, and nested `field_item` key scoping.
- Refine spec language by renaming Appendix B to broader recommendations and documenting custom vocabulary naming/namespacing guidance.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="23"/>
-    <col width="20" customWidth="1" style="1" min="24" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="25"/>
+    <col width="20" customWidth="1" style="1" min="26" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="1" t="b">
         <v>0</v>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Appendix B: Recommendations](#appendix-b-recommendations) for naming and namespacing guidance for custom vocabularies.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">

</xml_diff>

<commit_message>
add `<layer>`, document tokenization guidelines
- Add optional `<layer>` to the element head (spec & validator).
- Add token vocabulary guidance.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="25"/>
-    <col width="20" customWidth="1" style="1" min="26" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="29"/>
+    <col width="20" customWidth="1" style="1" min="30" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1544,8 +1544,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; serves for establishing a logical document component. This can be useful for capturing fragmented components, e.g. spanning multiple bounding boxes (e.g. cross-column) or pages, or for defining anchors for cross references.&lt;br/&gt;
-To capture a fragmented component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them</t>
+          <t>Optional part of the element head; serves for establishing a logical document component. This can be useful for capturing fragmented components, e.g. spanning multiple bounding boxes (e.g. cross-column) or pages, or for defining anchors for cross references. To capture a fragmented component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1848,7 +1847,11 @@
           <t>`&lt;layer&gt;`</t>
         </is>
       </c>
-      <c r="C34" s="5" t="n"/>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>The conceptual layer of the host element in the document.</t>
+        </is>
+      </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
@@ -1867,9 +1870,6 @@
         <v>0</v>
       </c>
       <c r="I34" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J34" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>`class`</t>
+          <t>`value`</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3885,7 +3885,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>{"body", "furniture", "background", "invisible", "notes"}</t>
+          <t>{"body", "background", "furniture"}</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The layer value: "body" is for the document's main content, "background" is for watermarks and other background components, while "furniture" is the fallback for any supplementary components not contributing to the document's main content, such as navigation or decorations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
allow full sem. body in `<picture>`, add `<tabular>` for chart tables
- Allow a full semantic body in `<picture>` (text, nested pictures, etc.) via XSD and Schematron updates
- Introduce `<tabular>` as the OTSL payload for `<picture class="chart">`, with `src` first and `tabular` immediately after when both are present
- Refresh `form-examples.md` from legacy `form`/`form_item`/`form_heading` to `field_region`/`field_item`/`field_heading`
- Add markdown XML-snippet validation (`utils/validate_markdown_snippets.py`, `tests/test_markdown_snippets.py`)
- Regenerate spec reference exports and fix the README CONTRIBUTING link

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="66640" yWindow="4520" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -38,6 +38,19 @@
     <font>
       <name val="Aptos Narrow"/>
       <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
@@ -62,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -87,6 +100,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -601,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -610,8 +629,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="29"/>
-    <col width="20" customWidth="1" style="1" min="30" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="31"/>
+    <col width="20" customWidth="1" style="1" min="32" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -816,7 +835,11 @@
           <t>`&lt;heading&gt;`</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Captures a document heading.</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -849,7 +872,11 @@
           <t>`&lt;footnote&gt;`</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Captures footnote content.</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -882,7 +909,11 @@
           <t>`&lt;page_header&gt;`</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Captures page header content (material repeated at the top of a page).</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -915,7 +946,11 @@
           <t>`&lt;page_footer&gt;`</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Captures page footer content (material repeated at the bottom of a page).</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1033,7 +1068,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows semantic elements. And additionally as the first element of the element body of `&lt;picture class="chart"&gt;`.</t>
+          <t>Any context that allows semantic elements.</t>
         </is>
       </c>
       <c r="E12" s="6" t="b">
@@ -1145,7 +1180,11 @@
           <t>`&lt;code&gt;`</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Appendix B: Recommendations](#appendix-b-recommendations)).</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1180,7 +1219,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Element body can generally only contain a `&lt;src&gt;`, for image bytes or reference. Additionally, in case of `&lt;picture class="chart"&gt;` (and only then) the element body may contain a `&lt;table&gt;`, in which case it must begin with it.</t>
+          <t>The element body begins with a picture-specific sequence, followed by content allowed in any other semantic element body. The picture-specific sequence is:&lt;ul&gt;&lt;li&gt;an optional `&lt;src&gt;` element&lt;/li&gt;&lt;li&gt;an optional `&lt;tabular&gt;` element (only allowed for `&lt;picture class="chart"&gt;`)&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1197,10 +1236,8 @@
       <c r="G16" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="1" t="inlineStr">
-        <is>
-          <t>Not allowed (except `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`)</t>
-        </is>
+      <c r="H16" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I16" s="1" t="b">
         <v>1</v>
@@ -1217,7 +1254,11 @@
           <t>`&lt;marker&gt;`</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Captures the visible glyph or identifier (e.g. number) of a marker, e.g. in the context of a list item.</t>
+        </is>
+      </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1287,7 +1328,11 @@
           <t>`&lt;field_heading&gt;`</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Field heading within a `&lt;field_region&gt;; analogous to `&lt;heading&gt;` but scoped to field structures.</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Can only be descendant of `&lt;field_region&gt;`.</t>
@@ -1475,7 +1520,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Can only be part of the element head of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E24" s="6" t="b">
@@ -1512,7 +1557,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E25" s="6" t="b">
@@ -1549,7 +1594,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E26" s="6" t="b">
@@ -1586,7 +1631,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E27" s="6" t="b">
@@ -1626,7 +1671,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;href&gt;`.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E28" s="6" t="b">
@@ -1663,7 +1708,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;xref&gt;`.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E29" s="6" t="b">
@@ -1700,7 +1745,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E30" s="6" t="b">
@@ -1740,7 +1785,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E31" s="6" t="b">
@@ -1777,7 +1822,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E32" s="6" t="b">
@@ -1814,7 +1859,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E33" s="6" t="b">
@@ -1854,7 +1899,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E34" s="6" t="b">
@@ -2107,7 +2152,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;picture&gt;`.</t>
+          <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`.</t>
         </is>
       </c>
       <c r="E41" s="6" t="b">
@@ -2123,7 +2168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" ht="17" customHeight="1">
+    <row r="42" ht="51" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
@@ -2131,27 +2176,36 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="n"/>
+          <t>`&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Structured tabular data. Uses the same cell model as `&lt;table&gt;`, but without an element head of its own.</t>
+        </is>
+      </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F42" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G42" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H42" s="1" t="b">
-        <v>0</v>
-      </c>
+          <t>Can only be part of the picture-specific element body sequence of [`&lt;picture class="chart"&gt;`](#picture).</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+        </is>
+      </c>
+      <c r="H42" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I42" s="10" t="n"/>
     </row>
     <row r="43" ht="17" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -2161,23 +2215,27 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>`&lt;content&gt;`</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="n"/>
+          <t>`&lt;checkbox&gt;`</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Empty element representing checkbox selection state.</t>
+        </is>
+      </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E43" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G43" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H43" s="1" t="b">
         <v>0</v>
@@ -2186,15 +2244,19 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="n"/>
+          <t>`&lt;content&gt;`</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Whitespace-preserving text container. Retains all whitespace within the element (equivalent to `xml:space="preserve"`), enabling use in whitespace-sensitive scenarios such as code blocks. XML special characters may alternatively be conveyed via CDATA.</t>
+        </is>
+      </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2206,7 +2268,7 @@
       <c r="F44" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G44" s="6" t="b">
+      <c r="G44" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="b">
@@ -2221,10 +2283,14 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="n"/>
+          <t>`&lt;bold&gt;`</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Indicates bold formatting.</t>
+        </is>
+      </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2251,10 +2317,14 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="n"/>
+          <t>`&lt;italic&gt;`</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Indicates italic formatting.</t>
+        </is>
+      </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2281,10 +2351,14 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="n"/>
+          <t>`&lt;underline&gt;`</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Indicates underlined formatting.</t>
+        </is>
+      </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2311,10 +2385,14 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="n"/>
+          <t>`&lt;strikethrough&gt;`</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Indicates struck-through formatting.</t>
+        </is>
+      </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2341,10 +2419,14 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="n"/>
+          <t>`&lt;superscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Indicates superscript formatting.</t>
+        </is>
+      </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2371,10 +2453,14 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="n"/>
+          <t>`&lt;subscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Indicates subscript formatting.</t>
+        </is>
+      </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2401,12 +2487,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
+          <t>`&lt;handwriting&gt;`</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Indicates right-to-left direction.</t>
+          <t>Indicates handwritten text.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2430,32 +2516,32 @@
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;rtl&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates right-to-left direction.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E52" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F52" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G52" s="1" t="b">
-        <v>0</v>
+      <c r="G52" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H52" s="1" t="b">
         <v>0</v>
@@ -2469,17 +2555,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
         </is>
       </c>
       <c r="E53" s="6" t="b">
@@ -2503,17 +2589,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
         </is>
       </c>
       <c r="E54" s="6" t="b">
@@ -2537,315 +2623,304 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
+          <t>`&lt;ched&gt;`</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a column header cell.</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H55" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" ht="17" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
           <t>`&lt;rhed&gt;`</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a row header cell.</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F55" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G55" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H55" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" ht="34" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H56" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" ht="34" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>`&lt;corn&gt;`</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F56" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G56" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H56" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" ht="17" customHeight="1">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G57" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H57" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>`&lt;srow&gt;`</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a section row header.</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F57" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G57" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H57" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" ht="51" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="51" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>`&lt;lcel&gt;`</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G58" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H58" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="34" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" ht="34" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>`&lt;ucel&gt;`</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" ht="51" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F60" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H60" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" ht="51" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F60" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G60" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H60" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" ht="17" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" ht="17" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>`&lt;nl&gt;`</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Denotes the end of a table row.</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H61" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" ht="34" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H62" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="34" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>`&lt;ldiv&gt;`</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;list&gt;`.</t>
         </is>
       </c>
-      <c r="E62" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F62" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G62" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H62" s="1" t="inlineStr">
+      <c r="E63" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F63" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G63" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H63" s="1" t="inlineStr">
         <is>
           <t>Only `&lt;marker&gt;`</t>
         </is>
-      </c>
-    </row>
-    <row r="63" ht="17" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>[07] document head</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;title&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J63" s="1" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
@@ -2856,7 +2931,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
+          <t>`&lt;title&gt;`</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2901,7 +2976,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2946,30 +3021,41 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F66" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G66" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H66" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J66" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="67" ht="17" customHeight="1">
@@ -2980,41 +3066,30 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J67" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H67" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3025,7 +3100,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3070,7 +3145,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -3115,7 +3190,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3160,7 +3235,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3205,7 +3280,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3250,7 +3325,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3295,7 +3370,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3340,7 +3415,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3385,7 +3460,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3430,7 +3505,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3475,7 +3550,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;access_policy&gt;`</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -3520,55 +3595,100 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
+          <t>`&lt;retention_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J79" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" ht="17" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
           <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J79" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="1" t="n"/>
-      <c r="B80" s="1" t="n"/>
-      <c r="C80" s="1" t="n"/>
-      <c r="D80" s="1" t="n"/>
-      <c r="F80" s="1" t="n"/>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="4" t="n"/>
+      <c r="A81" s="1" t="n"/>
+      <c r="B81" s="1" t="n"/>
+      <c r="C81" s="1" t="n"/>
+      <c r="D81" s="1" t="n"/>
+      <c r="F81" s="1" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H79"/>
+  <autoFilter ref="A1:H80"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3770,7 +3890,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Integer within [0, `location.resolution`)</t>
+          <t>Integer within [0, `location@resolution`)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3915,6 +4035,11 @@
           <t>Positive integer</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>The heading depth (1 = top-level).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3937,6 +4062,11 @@
           <t>{"read_only", "fillable"}</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>The value type.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3959,6 +4089,11 @@
           <t>{"unordered", "ordered"}</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>The list type.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4008,6 +4143,11 @@
           <t>{"unselected", "selected"}</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>The checkbox type.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4185,6 +4325,11 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>The field heading depth (1 = top-level).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
introduce archive format (#147)
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -629,8 +629,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="31"/>
-    <col width="20" customWidth="1" style="1" min="32" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="32"/>
+    <col width="20" customWidth="1" style="1" min="33" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Appendix B: Recommendations](#appendix-b-recommendations)).</t>
+          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Recommendations](#recommendations)).</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Appendix B: Recommendations](#appendix-b-recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">

</xml_diff>

<commit_message>
add `<description>` and `<summary>`
- Added optional `<description>` and `<summary>` elements to the element head in the spec documentation.
- Updated relevant sections in the XSD and Schematron to enforce the correct order of these elements.
- Update test suite accordingly
- Document diffences between `<caption>`, `<description>`, and `<summary>`
- Fix minor typo in recommended token vocabulary

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="66640" yWindow="4520" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -629,8 +629,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="32"/>
-    <col width="20" customWidth="1" style="1" min="33" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="36"/>
+    <col width="20" customWidth="1" style="1" min="37" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1515,7 +1515,8 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head for capturing an associated caption.</t>
+          <t>Optional part of the element head for capturing an associated caption. Unlike `&lt;description&gt;` or `&lt;summary&gt;`, `&lt;caption&gt;` is an actual
+document component, which can have its own location information etc. For example, a caption shown underneath a chart.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1775,12 +1776,14 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>`&lt;custom&gt;`</t>
+          <t>`&lt;description&gt;`</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+          <t>Optional part of the element head for capturing a derived textual account of what the host component is or what it shows. Unlike
+`&lt;caption&gt;`, `&lt;description&gt;` is meta-information and not an actual document component. For example, a picture
+description inferred by a model.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1795,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" s="1" t="b">
         <v>0</v>
@@ -1810,133 +1813,135 @@
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;summary&gt;`</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Optional part of the element head for capturing a derived textual distillation of what the host component conveys. Unlike
+`&lt;caption&gt;`, `&lt;summary&gt;` is meta-information and not part of the original document content.</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;custom&gt;`</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>`&lt;location&gt;`</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Optional part of the element head; coordinate system is the top-left corner of the page. When present, appears in sequence of 4 `&lt;location&gt;` instances, representing x0, y0, x1, y1. The following must then hold: `x0_norm&lt;=x1_norm` and `y0_norm&lt;=y1_norm`(i.e. first top-left point then bottom-right point), whereby `*_norm` is the respective coordinate normalized to its effective resolution.</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
-      <c r="E32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I32" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" ht="85" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="E34" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" ht="85" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>`&lt;timestamp&gt;`</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>TBD. Needed, if the individual hour/minute/etc are not all required (else cannot unambiguously interpret `&lt;hour&gt;0&lt;/hour&gt;&lt;minute&gt;2&lt;/minute&gt;&lt;second&gt;3&lt;/second&gt;`)</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
-      <c r="E33" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F33" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G33" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H33" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I33" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J33" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>[03a] property (outer)</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;layer&gt;`</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>The conceptual layer of the host element in the document.</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F34" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H34" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I34" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>[03b] property (inner)</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;hour&gt;`</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
       <c r="E35" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" s="6" t="b">
         <v>0</v>
@@ -1948,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" s="1" t="b">
         <v>1</v>
@@ -1957,18 +1962,22 @@
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>[03b] property (inner)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>`&lt;minute&gt;`</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="n"/>
+          <t>`&lt;layer&gt;`</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>The conceptual layer of the host element in the document.</t>
+        </is>
+      </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E36" s="6" t="b">
@@ -1984,9 +1993,6 @@
         <v>0</v>
       </c>
       <c r="I36" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J36" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1998,7 +2004,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>`&lt;second&gt;`</t>
+          <t>`&lt;hour&gt;`</t>
         </is>
       </c>
       <c r="C37" s="5" t="n"/>
@@ -2034,7 +2040,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>`&lt;centisecond&gt;`</t>
+          <t>`&lt;minute&gt;`</t>
         </is>
       </c>
       <c r="C38" s="5" t="n"/>
@@ -2070,23 +2076,23 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;second&gt;`</t>
         </is>
       </c>
       <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;meta&gt;`.</t>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
         </is>
       </c>
       <c r="E39" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G39" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" s="1" t="b">
         <v>0</v>
@@ -2106,189 +2112,193 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
+          <t>`&lt;centisecond&gt;`</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F40" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J40" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" ht="17" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>[03b] property (inner)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;summary&gt;`</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;meta&gt;`.</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G41" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>[03b] property (inner)</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
           <t>`&lt;classification&gt;`</t>
         </is>
       </c>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;meta&gt;`.</t>
         </is>
       </c>
-      <c r="E40" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G40" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H40" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I40" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J40" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" ht="34" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="E42" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G42" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>`&lt;src&gt;`</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>The image's source.</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`.</t>
         </is>
       </c>
-      <c r="E41" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F41" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G41" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H41" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" ht="51" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="E43" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G43" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H43" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="51" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>`&lt;tabular&gt;`</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Structured tabular data. Uses the same cell model as `&lt;table&gt;`, but without an element head of its own.</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Can only be part of the picture-specific element body sequence of [`&lt;picture class="chart"&gt;`](#picture).</t>
         </is>
       </c>
-      <c r="E42" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F42" s="10" t="inlineStr">
+      <c r="E44" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
         <is>
           <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
         </is>
       </c>
-      <c r="G42" s="10" t="inlineStr">
+      <c r="G44" s="10" t="inlineStr">
         <is>
           <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
         </is>
       </c>
-      <c r="H42" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I42" s="10" t="n"/>
-    </row>
-    <row r="43" ht="17" customHeight="1">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>[04] payload</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;checkbox&gt;`</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Empty element representing checkbox selection state.</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Any context that allows raw text content.</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F43" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G43" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H43" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" ht="17" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>[04] payload</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;content&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Whitespace-preserving text container. Retains all whitespace within the element (equivalent to `xml:space="preserve"`), enabling use in whitespace-sensitive scenarios such as code blocks. XML special characters may alternatively be conveyed via CDATA.</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Any context that allows raw text content.</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F44" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G44" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H44" s="1" t="b">
-        <v>0</v>
-      </c>
+      <c r="H44" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I44" s="10" t="n"/>
     </row>
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Indicates bold formatting.</t>
+          <t>Empty element representing checkbox selection state.</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -2297,13 +2307,13 @@
         </is>
       </c>
       <c r="E45" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F45" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G45" s="6" t="b">
-        <v>1</v>
+      <c r="G45" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H45" s="1" t="b">
         <v>0</v>
@@ -2312,17 +2322,17 @@
     <row r="46" ht="17" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
+          <t>`&lt;content&gt;`</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Indicates italic formatting.</t>
+          <t>Whitespace-preserving text container. Retains all whitespace within the element (equivalent to `xml:space="preserve"`), enabling use in whitespace-sensitive scenarios such as code blocks. XML special characters may alternatively be conveyed via CDATA.</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -2336,7 +2346,7 @@
       <c r="F46" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G46" s="6" t="b">
+      <c r="G46" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H46" s="1" t="b">
@@ -2351,12 +2361,12 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
+          <t>`&lt;bold&gt;`</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Indicates underlined formatting.</t>
+          <t>Indicates bold formatting.</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -2385,12 +2395,12 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
+          <t>`&lt;italic&gt;`</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Indicates struck-through formatting.</t>
+          <t>Indicates italic formatting.</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -2419,12 +2429,12 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
+          <t>`&lt;underline&gt;`</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Indicates superscript formatting.</t>
+          <t>Indicates underlined formatting.</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -2453,12 +2463,12 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
+          <t>`&lt;strikethrough&gt;`</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Indicates subscript formatting.</t>
+          <t>Indicates struck-through formatting.</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -2487,12 +2497,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
+          <t>`&lt;superscript&gt;`</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Indicates handwritten text.</t>
+          <t>Indicates superscript formatting.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2521,12 +2531,12 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
+          <t>`&lt;subscript&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates right-to-left direction.</t>
+          <t>Indicates subscript formatting.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -2550,32 +2560,32 @@
     <row r="53" ht="17" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;handwriting&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates handwritten text.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E53" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F53" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G53" s="1" t="b">
-        <v>0</v>
+      <c r="G53" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H53" s="1" t="b">
         <v>0</v>
@@ -2584,32 +2594,32 @@
     <row r="54" ht="17" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;rtl&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates right-to-left direction.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E54" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G54" s="1" t="b">
-        <v>0</v>
+      <c r="G54" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H54" s="1" t="b">
         <v>0</v>
@@ -2623,12 +2633,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2657,12 +2667,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rhed&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a row header cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2683,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" ht="34" customHeight="1">
+    <row r="57" ht="17" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2691,12 +2701,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>`&lt;corn&gt;`</t>
+          <t>`&lt;ched&gt;`</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+          <t>Indicates the beginning of a column header cell.</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2725,80 +2735,80 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
+          <t>`&lt;rhed&gt;`</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a row header cell.</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="34" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;corn&gt;`</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" ht="17" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
           <t>`&lt;srow&gt;`</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a section row header.</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G58" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H58" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="51" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;lcel&gt;`</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" ht="34" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;ucel&gt;`</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2827,89 +2837,89 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
+          <t>`&lt;lcel&gt;`</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" ht="34" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;ucel&gt;`</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H62" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="51" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
           <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
         </is>
       </c>
-      <c r="E61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H61" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" ht="17" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;nl&gt;`</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>Denotes the end of a table row.</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F62" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G62" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H62" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" ht="34" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;ldiv&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;list&gt;`.</t>
-        </is>
-      </c>
       <c r="E63" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F63" s="6" t="b">
         <v>0</v>
@@ -2917,100 +2927,78 @@
       <c r="G63" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H63" s="1" t="inlineStr">
-        <is>
-          <t>Only `&lt;marker&gt;`</t>
-        </is>
+      <c r="H63" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;title&gt;`</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J64" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" ht="17" customHeight="1">
+          <t>`&lt;nl&gt;`</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Denotes the end of a table row.</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G64" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H64" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" ht="34" customHeight="1">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J65" s="1" t="b">
-        <v>1</v>
+          <t>`&lt;ldiv&gt;`</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;list&gt;`.</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F65" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G65" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>Only `&lt;marker&gt;`</t>
+        </is>
       </c>
     </row>
     <row r="66" ht="17" customHeight="1">
@@ -3021,7 +3009,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;title&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -3066,30 +3054,41 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H67" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J67" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3100,7 +3099,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3145,41 +3144,30 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J69" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H69" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="70" ht="17" customHeight="1">
@@ -3190,7 +3178,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3235,7 +3223,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3280,7 +3268,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3325,7 +3313,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3370,7 +3358,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3415,7 +3403,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3460,7 +3448,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3505,7 +3493,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3550,7 +3538,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -3595,7 +3583,7 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -3640,55 +3628,145 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
+          <t>`&lt;access_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" ht="17" customHeight="1">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;retention_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J81" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" ht="17" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
           <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="n"/>
-      <c r="B81" s="1" t="n"/>
-      <c r="C81" s="1" t="n"/>
-      <c r="D81" s="1" t="n"/>
-      <c r="F81" s="1" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="n"/>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J82" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n"/>
+      <c r="B83" s="1" t="n"/>
+      <c r="C83" s="1" t="n"/>
+      <c r="D83" s="1" t="n"/>
+      <c r="F83" s="1" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H80"/>
+  <autoFilter ref="A1:H82"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
add `<description>` and `<summary>` (#150)
- Added optional `<description>` and `<summary>` elements to the element head in the spec documentation.
- Updated relevant sections in the XSD and Schematron to enforce the correct order of these elements.
- Update test suite accordingly
- Document diffences between `<caption>`, `<description>`, and `<summary>`
- Fix minor typo in recommended token vocabulary

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="66640" yWindow="4520" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -629,8 +629,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="32"/>
-    <col width="20" customWidth="1" style="1" min="33" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="36"/>
+    <col width="20" customWidth="1" style="1" min="37" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1515,7 +1515,8 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head for capturing an associated caption.</t>
+          <t>Optional part of the element head for capturing an associated caption. Unlike `&lt;description&gt;` or `&lt;summary&gt;`, `&lt;caption&gt;` is an actual
+document component, which can have its own location information etc. For example, a caption shown underneath a chart.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1775,12 +1776,14 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>`&lt;custom&gt;`</t>
+          <t>`&lt;description&gt;`</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+          <t>Optional part of the element head for capturing a derived textual account of what the host component is or what it shows. Unlike
+`&lt;caption&gt;`, `&lt;description&gt;` is meta-information and not an actual document component. For example, a picture
+description inferred by a model.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1795,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" s="1" t="b">
         <v>0</v>
@@ -1810,133 +1813,135 @@
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;summary&gt;`</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Optional part of the element head for capturing a derived textual distillation of what the host component conveys. Unlike
+`&lt;caption&gt;`, `&lt;summary&gt;` is meta-information and not part of the original document content.</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;custom&gt;`</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>`&lt;location&gt;`</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Optional part of the element head; coordinate system is the top-left corner of the page. When present, appears in sequence of 4 `&lt;location&gt;` instances, representing x0, y0, x1, y1. The following must then hold: `x0_norm&lt;=x1_norm` and `y0_norm&lt;=y1_norm`(i.e. first top-left point then bottom-right point), whereby `*_norm` is the respective coordinate normalized to its effective resolution.</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
-      <c r="E32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I32" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" ht="85" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="E34" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" ht="85" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>[03a] property (outer)</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>`&lt;timestamp&gt;`</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>TBD. Needed, if the individual hour/minute/etc are not all required (else cannot unambiguously interpret `&lt;hour&gt;0&lt;/hour&gt;&lt;minute&gt;2&lt;/minute&gt;&lt;second&gt;3&lt;/second&gt;`)</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
-      <c r="E33" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F33" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G33" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H33" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I33" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J33" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>[03a] property (outer)</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;layer&gt;`</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>The conceptual layer of the host element in the document.</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F34" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H34" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I34" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>[03b] property (inner)</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;hour&gt;`</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Can only be child of a semantic element.</t>
-        </is>
-      </c>
       <c r="E35" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" s="6" t="b">
         <v>0</v>
@@ -1948,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" s="1" t="b">
         <v>1</v>
@@ -1957,18 +1962,22 @@
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>[03b] property (inner)</t>
+          <t>[03a] property (outer)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>`&lt;minute&gt;`</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="n"/>
+          <t>`&lt;layer&gt;`</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>The conceptual layer of the host element in the document.</t>
+        </is>
+      </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E36" s="6" t="b">
@@ -1984,9 +1993,6 @@
         <v>0</v>
       </c>
       <c r="I36" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J36" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1998,7 +2004,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>`&lt;second&gt;`</t>
+          <t>`&lt;hour&gt;`</t>
         </is>
       </c>
       <c r="C37" s="5" t="n"/>
@@ -2034,7 +2040,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>`&lt;centisecond&gt;`</t>
+          <t>`&lt;minute&gt;`</t>
         </is>
       </c>
       <c r="C38" s="5" t="n"/>
@@ -2070,23 +2076,23 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;second&gt;`</t>
         </is>
       </c>
       <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;meta&gt;`.</t>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
         </is>
       </c>
       <c r="E39" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G39" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" s="1" t="b">
         <v>0</v>
@@ -2106,189 +2112,193 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
+          <t>`&lt;centisecond&gt;`</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Can only be child of a semantic element.</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F40" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J40" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" ht="17" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>[03b] property (inner)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;summary&gt;`</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;meta&gt;`.</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G41" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>[03b] property (inner)</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
           <t>`&lt;classification&gt;`</t>
         </is>
       </c>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;meta&gt;`.</t>
         </is>
       </c>
-      <c r="E40" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G40" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H40" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I40" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J40" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" ht="34" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="E42" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G42" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>`&lt;src&gt;`</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>The image's source.</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`.</t>
         </is>
       </c>
-      <c r="E41" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F41" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G41" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H41" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" ht="51" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="E43" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G43" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H43" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="51" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>`&lt;tabular&gt;`</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Structured tabular data. Uses the same cell model as `&lt;table&gt;`, but without an element head of its own.</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Can only be part of the picture-specific element body sequence of [`&lt;picture class="chart"&gt;`](#picture).</t>
         </is>
       </c>
-      <c r="E42" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F42" s="10" t="inlineStr">
+      <c r="E44" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
         <is>
           <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
         </is>
       </c>
-      <c r="G42" s="10" t="inlineStr">
+      <c r="G44" s="10" t="inlineStr">
         <is>
           <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
         </is>
       </c>
-      <c r="H42" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I42" s="10" t="n"/>
-    </row>
-    <row r="43" ht="17" customHeight="1">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>[04] payload</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;checkbox&gt;`</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Empty element representing checkbox selection state.</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Any context that allows raw text content.</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F43" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G43" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H43" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" ht="17" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>[04] payload</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;content&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Whitespace-preserving text container. Retains all whitespace within the element (equivalent to `xml:space="preserve"`), enabling use in whitespace-sensitive scenarios such as code blocks. XML special characters may alternatively be conveyed via CDATA.</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Any context that allows raw text content.</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F44" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G44" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H44" s="1" t="b">
-        <v>0</v>
-      </c>
+      <c r="H44" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I44" s="10" t="n"/>
     </row>
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
+          <t>`&lt;checkbox&gt;`</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Indicates bold formatting.</t>
+          <t>Empty element representing checkbox selection state.</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -2297,13 +2307,13 @@
         </is>
       </c>
       <c r="E45" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F45" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G45" s="6" t="b">
-        <v>1</v>
+      <c r="G45" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H45" s="1" t="b">
         <v>0</v>
@@ -2312,17 +2322,17 @@
     <row r="46" ht="17" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
+          <t>`&lt;content&gt;`</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Indicates italic formatting.</t>
+          <t>Whitespace-preserving text container. Retains all whitespace within the element (equivalent to `xml:space="preserve"`), enabling use in whitespace-sensitive scenarios such as code blocks. XML special characters may alternatively be conveyed via CDATA.</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -2336,7 +2346,7 @@
       <c r="F46" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G46" s="6" t="b">
+      <c r="G46" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H46" s="1" t="b">
@@ -2351,12 +2361,12 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
+          <t>`&lt;bold&gt;`</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Indicates underlined formatting.</t>
+          <t>Indicates bold formatting.</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -2385,12 +2395,12 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
+          <t>`&lt;italic&gt;`</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Indicates struck-through formatting.</t>
+          <t>Indicates italic formatting.</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -2419,12 +2429,12 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
+          <t>`&lt;underline&gt;`</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Indicates superscript formatting.</t>
+          <t>Indicates underlined formatting.</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -2453,12 +2463,12 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
+          <t>`&lt;strikethrough&gt;`</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Indicates subscript formatting.</t>
+          <t>Indicates struck-through formatting.</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -2487,12 +2497,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
+          <t>`&lt;superscript&gt;`</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Indicates handwritten text.</t>
+          <t>Indicates superscript formatting.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2521,12 +2531,12 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
+          <t>`&lt;subscript&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates right-to-left direction.</t>
+          <t>Indicates subscript formatting.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -2550,32 +2560,32 @@
     <row r="53" ht="17" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;handwriting&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates handwritten text.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E53" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F53" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G53" s="1" t="b">
-        <v>0</v>
+      <c r="G53" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H53" s="1" t="b">
         <v>0</v>
@@ -2584,32 +2594,32 @@
     <row r="54" ht="17" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;rtl&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates right-to-left direction.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E54" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G54" s="1" t="b">
-        <v>0</v>
+      <c r="G54" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H54" s="1" t="b">
         <v>0</v>
@@ -2623,12 +2633,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2657,12 +2667,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rhed&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a row header cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2683,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" ht="34" customHeight="1">
+    <row r="57" ht="17" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2691,12 +2701,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>`&lt;corn&gt;`</t>
+          <t>`&lt;ched&gt;`</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+          <t>Indicates the beginning of a column header cell.</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2725,80 +2735,80 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
+          <t>`&lt;rhed&gt;`</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a row header cell.</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="34" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;corn&gt;`</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" ht="17" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
           <t>`&lt;srow&gt;`</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a section row header.</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G58" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H58" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="51" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;lcel&gt;`</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" ht="34" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;ucel&gt;`</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2827,89 +2837,89 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
+          <t>`&lt;lcel&gt;`</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" ht="34" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;ucel&gt;`</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H62" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="51" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
           <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
         </is>
       </c>
-      <c r="E61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H61" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" ht="17" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;nl&gt;`</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>Denotes the end of a table row.</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F62" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G62" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H62" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" ht="34" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>[06] structural</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;ldiv&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;list&gt;`.</t>
-        </is>
-      </c>
       <c r="E63" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F63" s="6" t="b">
         <v>0</v>
@@ -2917,100 +2927,78 @@
       <c r="G63" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H63" s="1" t="inlineStr">
-        <is>
-          <t>Only `&lt;marker&gt;`</t>
-        </is>
+      <c r="H63" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;title&gt;`</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J64" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" ht="17" customHeight="1">
+          <t>`&lt;nl&gt;`</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Denotes the end of a table row.</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F64" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G64" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H64" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" ht="34" customHeight="1">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>[07] document head</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J65" s="1" t="b">
-        <v>1</v>
+          <t>`&lt;ldiv&gt;`</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;list&gt;`.</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F65" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G65" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>Only `&lt;marker&gt;`</t>
+        </is>
       </c>
     </row>
     <row r="66" ht="17" customHeight="1">
@@ -3021,7 +3009,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;title&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -3066,30 +3054,41 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H67" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J67" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3100,7 +3099,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3145,41 +3144,30 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J69" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H69" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="70" ht="17" customHeight="1">
@@ -3190,7 +3178,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3235,7 +3223,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3280,7 +3268,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3325,7 +3313,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3370,7 +3358,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3415,7 +3403,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3460,7 +3448,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3505,7 +3493,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3550,7 +3538,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -3595,7 +3583,7 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -3640,55 +3628,145 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
+          <t>`&lt;access_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" ht="17" customHeight="1">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>`&lt;retention_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J81" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" ht="17" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
           <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="n"/>
-      <c r="B81" s="1" t="n"/>
-      <c r="C81" s="1" t="n"/>
-      <c r="D81" s="1" t="n"/>
-      <c r="F81" s="1" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="n"/>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J82" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n"/>
+      <c r="B83" s="1" t="n"/>
+      <c r="C83" s="1" t="n"/>
+      <c r="D83" s="1" t="n"/>
+      <c r="F83" s="1" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H80"/>
+  <autoFilter ref="A1:H82"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
prepare release v0.7.0 (#152)
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3855,12 +3855,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Optional; default: "0.6"</t>
+          <t>Optional; default: "0.7"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"0.6"}</t>
+          <t>{"0.7"}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
add track `<cover>`; make timestamp `<minutes>` optional
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -3613,56 +3613,56 @@
       </c>
     </row>
     <row r="79" ht="17" customHeight="1">
-      <c r="A79" s="4" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>[01b] semantic (inner)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
+          <t>`&lt;cover&gt;`</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>A representative image for a `&lt;track&gt;` as a whole — podcast artwork, a poster, a title card. Appears once, before the first cue block. Same shape as `&lt;frame&gt;`: an optional element head followed by an optional `&lt;src&gt;`.</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Can only appear inside a `&lt;track&gt;`, before the first `&lt;bdiv&gt;`.</t>
+        </is>
+      </c>
+      <c r="E79" t="b">
+        <v>1</v>
+      </c>
+      <c r="F79" t="b">
+        <v>1</v>
+      </c>
+      <c r="G79" t="b">
+        <v>0</v>
+      </c>
+      <c r="H79" t="b">
+        <v>1</v>
+      </c>
+      <c r="I79" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" ht="17" customHeight="1">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>[01b] semantic (inner)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>`&lt;frame&gt;`</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>The still image of the recording at a `&lt;track&gt;` cue block's start time. Shaped like `&lt;picture&gt;`: an optional element head followed by an optional `&lt;src&gt;`.</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Can only appear inside a `&lt;track&gt;` cue block.</t>
-        </is>
-      </c>
-      <c r="E79" t="b">
-        <v>1</v>
-      </c>
-      <c r="F79" t="b">
-        <v>1</v>
-      </c>
-      <c r="G79" t="b">
-        <v>0</v>
-      </c>
-      <c r="H79" t="b">
-        <v>1</v>
-      </c>
-      <c r="I79" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" ht="17" customHeight="1">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>[01b] semantic (inner)</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>`&lt;audio&gt;`</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>The recording over a `&lt;track&gt;` cue block's interval `[start, end]` — a temporal crop of the track's audio, as a `&lt;picture&gt;` crop corresponds to its page region. Requires the cue block to carry an end time; the timestamps are authoritative and the clip is a best-effort fragment. Same shape as `&lt;frame&gt;`.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3694,12 +3694,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>`&lt;voice&gt;`</t>
+          <t>`&lt;audio&gt;`</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Speaker attribution for a transcript turn within a `&lt;track&gt;` cue block. Handled like `&lt;text&gt;` (may carry its own element head and inline formatting).</t>
+          <t>The recording over a `&lt;track&gt;` cue block's interval `[start, end]` — a temporal crop of the track's audio, as a `&lt;picture&gt;` crop corresponds to its page region. Requires the cue block to carry an end time; the timestamps are authoritative and the clip is a best-effort fragment. Same shape as `&lt;frame&gt;`.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3714,7 +3714,7 @@
         <v>1</v>
       </c>
       <c r="G81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H81" t="b">
         <v>1</v>
@@ -3731,17 +3731,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>`&lt;chapter&gt;`</t>
+          <t>`&lt;voice&gt;`</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A chapter or section title for a `&lt;track&gt;`. It marks a chapter boundary at the start time of the cue block that carries it; the chapter runs until the next `&lt;chapter&gt;` (or `&lt;/track&gt;`), and the region before the first `&lt;chapter&gt;` is unchaptered. Only the start time matters — the cue block's end time bounds its transcript, not the chapter. Chapters form a flat partition (no nesting, no overlap). Handled like `&lt;text&gt;` (may carry its own element head and inline formatting).</t>
+          <t>Speaker attribution for a transcript turn within a `&lt;track&gt;` cue block. Handled like `&lt;text&gt;` (may carry its own element head and inline formatting).</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Can only appear inside a `&lt;track&gt;` cue block, after the start (and optional end) timestamp and before any `&lt;frame&gt;`.</t>
+          <t>Can only appear inside a `&lt;track&gt;` cue block.</t>
         </is>
       </c>
       <c r="E82" t="b">
@@ -3763,56 +3763,59 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[01b] semantic (inner)</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>`&lt;bdiv&gt;`</t>
+          <t>`&lt;chapter&gt;`</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a `&lt;track&gt;` cue block.</t>
+          <t>A chapter or section title for a `&lt;track&gt;`. It marks a chapter boundary at the start time of the cue block that carries it; the chapter runs until the next `&lt;chapter&gt;` (or `&lt;/track&gt;`), and the region before the first `&lt;chapter&gt;` is unchaptered. Only the start time matters — the cue block's end time bounds its transcript, not the chapter. Chapters form a flat partition (no nesting, no overlap). Handled like `&lt;text&gt;` (may carry its own element head and inline formatting).</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Can only be a child of `&lt;track&gt;`.</t>
+          <t>Can only appear inside a `&lt;track&gt;` cue block, after the start (and optional end) timestamp and before any `&lt;frame&gt;`.</t>
         </is>
       </c>
       <c r="E83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H83" t="b">
+        <v>1</v>
+      </c>
+      <c r="I83" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>[04] payload</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>`&lt;hours&gt;`</t>
+          <t>`&lt;bdiv&gt;`</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Hours component of a `&lt;track&gt;` cue timestamp. Optional within a timestamp run (defaults to 0).</t>
+          <t>Indicates the beginning of a `&lt;track&gt;` cue block.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Can only be part of a timestamp run in a `&lt;track&gt;` cue block.</t>
+          <t>Can only be a child of `&lt;track&gt;`.</t>
         </is>
       </c>
       <c r="E84" t="b">
@@ -3836,12 +3839,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>`&lt;minutes&gt;`</t>
+          <t>`&lt;hours&gt;`</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Minutes component of a `&lt;track&gt;` cue timestamp.</t>
+          <t>Hours component of a `&lt;track&gt;` cue timestamp. Optional within a timestamp run (defaults to 0).</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3870,12 +3873,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>`&lt;seconds&gt;`</t>
+          <t>`&lt;minutes&gt;`</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Seconds component of a `&lt;track&gt;` cue timestamp.</t>
+          <t>Minutes component of a `&lt;track&gt;` cue timestamp. Optional within a timestamp run (defaults to 0).</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3904,29 +3907,63 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
+          <t>`&lt;seconds&gt;`</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Seconds component of a `&lt;track&gt;` cue timestamp.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Can only be part of a timestamp run in a `&lt;track&gt;` cue block.</t>
+        </is>
+      </c>
+      <c r="E87" t="b">
+        <v>0</v>
+      </c>
+      <c r="F87" t="b">
+        <v>0</v>
+      </c>
+      <c r="G87" t="b">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>[04] payload</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>`&lt;msecs&gt;`</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Milliseconds component of a `&lt;track&gt;` cue timestamp. Optional within a timestamp run (defaults to 0).</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>Can only be part of a timestamp run in a `&lt;track&gt;` cue block.</t>
         </is>
       </c>
-      <c r="E87" t="b">
-        <v>0</v>
-      </c>
-      <c r="F87" t="b">
-        <v>0</v>
-      </c>
-      <c r="G87" t="b">
-        <v>0</v>
-      </c>
-      <c r="H87" t="b">
+      <c r="E88" t="b">
+        <v>0</v>
+      </c>
+      <c r="F88" t="b">
+        <v>0</v>
+      </c>
+      <c r="G88" t="b">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>